<commit_message>
salvo antes do patch
</commit_message>
<xml_diff>
--- a/analisesFinais.xlsx
+++ b/analisesFinais.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PolyanaSilva\Documents\BP_VRPTW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF2D868-B4BD-4D03-A2F3-B71ECD0C6E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D42FFD7-3FC2-478A-90EF-7FF56D17ED05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{E7DF56F7-393C-4179-80B5-2006709A41FF}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="4" xr2:uid="{E7DF56F7-393C-4179-80B5-2006709A41FF}"/>
   </bookViews>
   <sheets>
     <sheet name="PRICING25" sheetId="2" r:id="rId1"/>
     <sheet name="SM25" sheetId="3" r:id="rId2"/>
     <sheet name="Análise_25nósComSemEstabIntegGe" sheetId="5" r:id="rId3"/>
-    <sheet name="FO_CONHECIDA" sheetId="4" r:id="rId4"/>
-    <sheet name="Construtiva50" sheetId="6" r:id="rId5"/>
+    <sheet name="Construtiva50" sheetId="6" r:id="rId4"/>
+    <sheet name="50SM20" sheetId="7" r:id="rId5"/>
+    <sheet name="FO_CONHECIDA" sheetId="4" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PRICING25!$A$1:$V$117</definedName>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1467" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1514" uniqueCount="510">
   <si>
     <t>run_id</t>
   </si>
@@ -1522,6 +1523,60 @@
   </si>
   <si>
     <t>Construtiva 50</t>
+  </si>
+  <si>
+    <t>902.80</t>
+  </si>
+  <si>
+    <t>888.70</t>
+  </si>
+  <si>
+    <t>711.10</t>
+  </si>
+  <si>
+    <t>763.80</t>
+  </si>
+  <si>
+    <t>876.80</t>
+  </si>
+  <si>
+    <t>900.80</t>
+  </si>
+  <si>
+    <t>784.80</t>
+  </si>
+  <si>
+    <t>734.30</t>
+  </si>
+  <si>
+    <t>1034.50</t>
+  </si>
+  <si>
+    <t>737.80</t>
+  </si>
+  <si>
+    <t>768.30</t>
+  </si>
+  <si>
+    <t>545.80</t>
+  </si>
+  <si>
+    <t>883.30</t>
+  </si>
+  <si>
+    <t>770.00</t>
+  </si>
+  <si>
+    <t>721.90</t>
+  </si>
+  <si>
+    <t>638.40</t>
+  </si>
+  <si>
+    <t>Inst</t>
+  </si>
+  <si>
+    <t>FoConhecido</t>
   </si>
 </sst>
 </file>
@@ -2201,36 +2256,6 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="21" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2260,6 +2285,36 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="20" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -13033,10 +13088,10 @@
   <dimension ref="A1:X106"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.21875" style="3" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="12.88671875" customWidth="1"/>
@@ -13121,15 +13176,15 @@
       <c r="M2">
         <v>78.450450897216797</v>
       </c>
-      <c r="R2" s="91" t="s">
+      <c r="R2" s="101" t="s">
         <v>220</v>
       </c>
-      <c r="S2" s="92"/>
-      <c r="T2" s="92"/>
-      <c r="U2" s="92"/>
-      <c r="V2" s="92"/>
-      <c r="W2" s="92"/>
-      <c r="X2" s="92"/>
+      <c r="S2" s="102"/>
+      <c r="T2" s="102"/>
+      <c r="U2" s="102"/>
+      <c r="V2" s="102"/>
+      <c r="W2" s="102"/>
+      <c r="X2" s="102"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -17430,61 +17485,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:18" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="98" t="s">
+      <c r="B1" s="104" t="s">
         <v>346</v>
       </c>
-      <c r="C1" s="98"/>
-      <c r="D1" s="98"/>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="98"/>
-      <c r="I1" s="98"/>
-      <c r="J1" s="98"/>
-      <c r="K1" s="98"/>
-      <c r="L1" s="98"/>
-      <c r="M1" s="98"/>
-      <c r="N1" s="98"/>
-      <c r="O1" s="98"/>
-      <c r="P1" s="98"/>
-      <c r="Q1" s="98"/>
-      <c r="R1" s="98"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="104"/>
+      <c r="L1" s="104"/>
+      <c r="M1" s="104"/>
+      <c r="N1" s="104"/>
+      <c r="O1" s="104"/>
+      <c r="P1" s="104"/>
+      <c r="Q1" s="104"/>
+      <c r="R1" s="104"/>
     </row>
     <row r="2" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="99" t="s">
+      <c r="B2" s="105" t="s">
         <v>347</v>
       </c>
-      <c r="C2" s="99"/>
-      <c r="D2" s="99"/>
-      <c r="E2" s="99"/>
-      <c r="F2" s="99"/>
-      <c r="G2" s="99"/>
-      <c r="H2" s="99"/>
-      <c r="I2" s="99"/>
-      <c r="J2" s="99"/>
-      <c r="K2" s="99"/>
-      <c r="L2" s="99"/>
-      <c r="M2" s="99"/>
-      <c r="N2" s="99"/>
-      <c r="O2" s="99"/>
-      <c r="P2" s="99"/>
-      <c r="Q2" s="99"/>
-      <c r="R2" s="99"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="105"/>
+      <c r="L2" s="105"/>
+      <c r="M2" s="105"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="105"/>
+      <c r="P2" s="105"/>
+      <c r="Q2" s="105"/>
+      <c r="R2" s="105"/>
     </row>
     <row r="4" spans="2:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="94" t="s">
+      <c r="B4" s="103" t="s">
         <v>348</v>
       </c>
-      <c r="C4" s="94"/>
-      <c r="D4" s="94"/>
-      <c r="E4" s="94"/>
-      <c r="F4" s="94"/>
-      <c r="G4" s="94"/>
-      <c r="H4" s="94"/>
-      <c r="I4" s="94"/>
-      <c r="J4" s="94"/>
-      <c r="K4" s="94"/>
-      <c r="L4" s="94"/>
+      <c r="C4" s="103"/>
+      <c r="D4" s="103"/>
+      <c r="E4" s="103"/>
+      <c r="F4" s="103"/>
+      <c r="G4" s="103"/>
+      <c r="H4" s="103"/>
+      <c r="I4" s="103"/>
+      <c r="J4" s="103"/>
+      <c r="K4" s="103"/>
+      <c r="L4" s="103"/>
     </row>
     <row r="5" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="22" t="s">
@@ -17640,124 +17695,124 @@
       <c r="L9" s="41"/>
     </row>
     <row r="11" spans="2:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="100" t="s">
+      <c r="B11" s="106" t="s">
         <v>369</v>
       </c>
-      <c r="C11" s="100"/>
-      <c r="D11" s="100"/>
-      <c r="E11" s="100"/>
-      <c r="F11" s="100"/>
-      <c r="G11" s="100"/>
-      <c r="H11" s="100"/>
-      <c r="I11" s="100"/>
-      <c r="J11" s="100"/>
-      <c r="K11" s="100"/>
-      <c r="L11" s="100"/>
+      <c r="C11" s="106"/>
+      <c r="D11" s="106"/>
+      <c r="E11" s="106"/>
+      <c r="F11" s="106"/>
+      <c r="G11" s="106"/>
+      <c r="H11" s="106"/>
+      <c r="I11" s="106"/>
+      <c r="J11" s="106"/>
+      <c r="K11" s="106"/>
+      <c r="L11" s="106"/>
     </row>
     <row r="12" spans="2:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="22" t="s">
         <v>370</v>
       </c>
-      <c r="C12" s="95" t="s">
+      <c r="C12" s="107" t="s">
         <v>371</v>
       </c>
-      <c r="D12" s="95"/>
-      <c r="E12" s="95"/>
-      <c r="F12" s="95"/>
-      <c r="G12" s="95"/>
-      <c r="H12" s="95"/>
-      <c r="I12" s="95"/>
-      <c r="J12" s="95"/>
-      <c r="K12" s="95"/>
-      <c r="L12" s="95"/>
+      <c r="D12" s="107"/>
+      <c r="E12" s="107"/>
+      <c r="F12" s="107"/>
+      <c r="G12" s="107"/>
+      <c r="H12" s="107"/>
+      <c r="I12" s="107"/>
+      <c r="J12" s="107"/>
+      <c r="K12" s="107"/>
+      <c r="L12" s="107"/>
     </row>
     <row r="13" spans="2:18" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="46" t="s">
         <v>372</v>
       </c>
-      <c r="C13" s="97" t="s">
+      <c r="C13" s="108" t="s">
         <v>373</v>
       </c>
-      <c r="D13" s="97"/>
-      <c r="E13" s="97"/>
-      <c r="F13" s="97"/>
-      <c r="G13" s="97"/>
-      <c r="H13" s="97"/>
-      <c r="I13" s="97"/>
-      <c r="J13" s="97"/>
-      <c r="K13" s="97"/>
-      <c r="L13" s="97"/>
+      <c r="D13" s="108"/>
+      <c r="E13" s="108"/>
+      <c r="F13" s="108"/>
+      <c r="G13" s="108"/>
+      <c r="H13" s="108"/>
+      <c r="I13" s="108"/>
+      <c r="J13" s="108"/>
+      <c r="K13" s="108"/>
+      <c r="L13" s="108"/>
     </row>
     <row r="14" spans="2:18" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="47" t="s">
         <v>374</v>
       </c>
-      <c r="C14" s="96" t="s">
+      <c r="C14" s="109" t="s">
         <v>375</v>
       </c>
-      <c r="D14" s="96"/>
-      <c r="E14" s="96"/>
-      <c r="F14" s="96"/>
-      <c r="G14" s="96"/>
-      <c r="H14" s="96"/>
-      <c r="I14" s="96"/>
-      <c r="J14" s="96"/>
-      <c r="K14" s="96"/>
-      <c r="L14" s="96"/>
+      <c r="D14" s="109"/>
+      <c r="E14" s="109"/>
+      <c r="F14" s="109"/>
+      <c r="G14" s="109"/>
+      <c r="H14" s="109"/>
+      <c r="I14" s="109"/>
+      <c r="J14" s="109"/>
+      <c r="K14" s="109"/>
+      <c r="L14" s="109"/>
     </row>
     <row r="15" spans="2:18" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="46" t="s">
         <v>376</v>
       </c>
-      <c r="C15" s="97" t="s">
+      <c r="C15" s="108" t="s">
         <v>377</v>
       </c>
-      <c r="D15" s="97"/>
-      <c r="E15" s="97"/>
-      <c r="F15" s="97"/>
-      <c r="G15" s="97"/>
-      <c r="H15" s="97"/>
-      <c r="I15" s="97"/>
-      <c r="J15" s="97"/>
-      <c r="K15" s="97"/>
-      <c r="L15" s="97"/>
+      <c r="D15" s="108"/>
+      <c r="E15" s="108"/>
+      <c r="F15" s="108"/>
+      <c r="G15" s="108"/>
+      <c r="H15" s="108"/>
+      <c r="I15" s="108"/>
+      <c r="J15" s="108"/>
+      <c r="K15" s="108"/>
+      <c r="L15" s="108"/>
     </row>
     <row r="16" spans="2:18" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="47" t="s">
         <v>378</v>
       </c>
-      <c r="C16" s="96" t="s">
+      <c r="C16" s="109" t="s">
         <v>379</v>
       </c>
-      <c r="D16" s="96"/>
-      <c r="E16" s="96"/>
-      <c r="F16" s="96"/>
-      <c r="G16" s="96"/>
-      <c r="H16" s="96"/>
-      <c r="I16" s="96"/>
-      <c r="J16" s="96"/>
-      <c r="K16" s="96"/>
-      <c r="L16" s="96"/>
+      <c r="D16" s="109"/>
+      <c r="E16" s="109"/>
+      <c r="F16" s="109"/>
+      <c r="G16" s="109"/>
+      <c r="H16" s="109"/>
+      <c r="I16" s="109"/>
+      <c r="J16" s="109"/>
+      <c r="K16" s="109"/>
+      <c r="L16" s="109"/>
     </row>
     <row r="18" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="94" t="s">
+      <c r="B18" s="103" t="s">
         <v>380</v>
       </c>
-      <c r="C18" s="94"/>
-      <c r="D18" s="94"/>
-      <c r="E18" s="94"/>
-      <c r="F18" s="94"/>
-      <c r="G18" s="94"/>
-      <c r="H18" s="94"/>
-      <c r="I18" s="94"/>
-      <c r="J18" s="94"/>
-      <c r="K18" s="94"/>
-      <c r="L18" s="94"/>
-      <c r="M18" s="94"/>
-      <c r="N18" s="94"/>
-      <c r="O18" s="94"/>
-      <c r="P18" s="94"/>
-      <c r="Q18" s="94"/>
+      <c r="C18" s="103"/>
+      <c r="D18" s="103"/>
+      <c r="E18" s="103"/>
+      <c r="F18" s="103"/>
+      <c r="G18" s="103"/>
+      <c r="H18" s="103"/>
+      <c r="I18" s="103"/>
+      <c r="J18" s="103"/>
+      <c r="K18" s="103"/>
+      <c r="L18" s="103"/>
+      <c r="M18" s="103"/>
+      <c r="N18" s="103"/>
+      <c r="O18" s="103"/>
+      <c r="P18" s="103"/>
+      <c r="Q18" s="103"/>
     </row>
     <row r="19" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="22" t="s">
@@ -18079,19 +18134,19 @@
       <c r="H35" s="61"/>
     </row>
     <row r="37" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="94" t="s">
+      <c r="B37" s="103" t="s">
         <v>393</v>
       </c>
-      <c r="C37" s="94"/>
-      <c r="D37" s="94"/>
-      <c r="E37" s="94"/>
-      <c r="F37" s="94"/>
-      <c r="G37" s="94"/>
-      <c r="H37" s="94"/>
-      <c r="I37" s="94"/>
-      <c r="J37" s="94"/>
-      <c r="K37" s="94"/>
-      <c r="L37" s="94"/>
+      <c r="C37" s="103"/>
+      <c r="D37" s="103"/>
+      <c r="E37" s="103"/>
+      <c r="F37" s="103"/>
+      <c r="G37" s="103"/>
+      <c r="H37" s="103"/>
+      <c r="I37" s="103"/>
+      <c r="J37" s="103"/>
+      <c r="K37" s="103"/>
+      <c r="L37" s="103"/>
     </row>
     <row r="38" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="22" t="s">
@@ -18360,15 +18415,15 @@
       <c r="I50" s="61"/>
     </row>
     <row r="52" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="94" t="s">
+      <c r="B52" s="103" t="s">
         <v>398</v>
       </c>
-      <c r="C52" s="94"/>
-      <c r="D52" s="94"/>
-      <c r="E52" s="94"/>
-      <c r="F52" s="94"/>
-      <c r="G52" s="94"/>
-      <c r="H52" s="94"/>
+      <c r="C52" s="103"/>
+      <c r="D52" s="103"/>
+      <c r="E52" s="103"/>
+      <c r="F52" s="103"/>
+      <c r="G52" s="103"/>
+      <c r="H52" s="103"/>
     </row>
     <row r="53" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="22" t="s">
@@ -18456,15 +18511,15 @@
       </c>
     </row>
     <row r="60" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="94" t="s">
+      <c r="B60" s="103" t="s">
         <v>400</v>
       </c>
-      <c r="C60" s="94"/>
-      <c r="D60" s="94"/>
-      <c r="E60" s="94"/>
-      <c r="F60" s="94"/>
-      <c r="G60" s="94"/>
-      <c r="H60" s="94"/>
+      <c r="C60" s="103"/>
+      <c r="D60" s="103"/>
+      <c r="E60" s="103"/>
+      <c r="F60" s="103"/>
+      <c r="G60" s="103"/>
+      <c r="H60" s="103"/>
     </row>
     <row r="61" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="22" t="s">
@@ -18627,15 +18682,15 @@
       </c>
     </row>
     <row r="68" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="94" t="s">
+      <c r="B68" s="103" t="s">
         <v>401</v>
       </c>
-      <c r="C68" s="94"/>
-      <c r="D68" s="94"/>
-      <c r="E68" s="94"/>
-      <c r="F68" s="94"/>
-      <c r="G68" s="94"/>
-      <c r="H68" s="94"/>
+      <c r="C68" s="103"/>
+      <c r="D68" s="103"/>
+      <c r="E68" s="103"/>
+      <c r="F68" s="103"/>
+      <c r="G68" s="103"/>
+      <c r="H68" s="103"/>
     </row>
     <row r="69" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="22" t="s">
@@ -18758,60 +18813,67 @@
       </c>
     </row>
     <row r="77" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="95" t="s">
+      <c r="B77" s="107" t="s">
         <v>410</v>
       </c>
-      <c r="C77" s="95"/>
-      <c r="D77" s="95"/>
-      <c r="E77" s="95"/>
-      <c r="F77" s="95"/>
+      <c r="C77" s="107"/>
+      <c r="D77" s="107"/>
+      <c r="E77" s="107"/>
+      <c r="F77" s="107"/>
     </row>
     <row r="78" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B78" s="48" t="s">
         <v>386</v>
       </c>
-      <c r="C78" s="93" t="s">
+      <c r="C78" s="110" t="s">
         <v>359</v>
       </c>
-      <c r="D78" s="93"/>
-      <c r="E78" s="93"/>
-      <c r="F78" s="93"/>
+      <c r="D78" s="110"/>
+      <c r="E78" s="110"/>
+      <c r="F78" s="110"/>
     </row>
     <row r="79" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B79" s="49" t="s">
         <v>389</v>
       </c>
-      <c r="C79" s="93" t="s">
+      <c r="C79" s="110" t="s">
         <v>361</v>
       </c>
-      <c r="D79" s="93"/>
-      <c r="E79" s="93"/>
-      <c r="F79" s="93"/>
+      <c r="D79" s="110"/>
+      <c r="E79" s="110"/>
+      <c r="F79" s="110"/>
     </row>
     <row r="80" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B80" s="50" t="s">
         <v>394</v>
       </c>
-      <c r="C80" s="93" t="s">
+      <c r="C80" s="110" t="s">
         <v>366</v>
       </c>
-      <c r="D80" s="93"/>
-      <c r="E80" s="93"/>
-      <c r="F80" s="93"/>
+      <c r="D80" s="110"/>
+      <c r="E80" s="110"/>
+      <c r="F80" s="110"/>
     </row>
     <row r="81" spans="2:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B81" s="51" t="s">
         <v>396</v>
       </c>
-      <c r="C81" s="93" t="s">
+      <c r="C81" s="110" t="s">
         <v>368</v>
       </c>
-      <c r="D81" s="93"/>
-      <c r="E81" s="93"/>
-      <c r="F81" s="93"/>
+      <c r="D81" s="110"/>
+      <c r="E81" s="110"/>
+      <c r="F81" s="110"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="C81:F81"/>
+    <mergeCell ref="B60:H60"/>
+    <mergeCell ref="B68:H68"/>
+    <mergeCell ref="B77:F77"/>
+    <mergeCell ref="C78:F78"/>
+    <mergeCell ref="C79:F79"/>
+    <mergeCell ref="C80:F80"/>
     <mergeCell ref="B52:H52"/>
     <mergeCell ref="B1:R1"/>
     <mergeCell ref="B2:R2"/>
@@ -18824,13 +18886,6 @@
     <mergeCell ref="C16:L16"/>
     <mergeCell ref="B18:Q18"/>
     <mergeCell ref="B37:L37"/>
-    <mergeCell ref="C81:F81"/>
-    <mergeCell ref="B60:H60"/>
-    <mergeCell ref="B68:H68"/>
-    <mergeCell ref="B77:F77"/>
-    <mergeCell ref="C78:F78"/>
-    <mergeCell ref="C79:F79"/>
-    <mergeCell ref="C80:F80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -18839,6 +18894,1068 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6381B92-E053-4233-81A5-0B655C210782}">
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>446</v>
+      </c>
+      <c r="B1" t="s">
+        <v>447</v>
+      </c>
+      <c r="C1" t="s">
+        <v>448</v>
+      </c>
+      <c r="D1" t="s">
+        <v>449</v>
+      </c>
+      <c r="E1" t="s">
+        <v>447</v>
+      </c>
+      <c r="F1">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s">
+        <v>450</v>
+      </c>
+      <c r="H1" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D2" t="s">
+        <v>452</v>
+      </c>
+      <c r="E2" t="s">
+        <v>447</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s">
+        <v>450</v>
+      </c>
+      <c r="H2" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>241</v>
+      </c>
+      <c r="B3" t="s">
+        <v>447</v>
+      </c>
+      <c r="C3" t="s">
+        <v>448</v>
+      </c>
+      <c r="D3" t="s">
+        <v>453</v>
+      </c>
+      <c r="E3" t="s">
+        <v>447</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
+        <v>450</v>
+      </c>
+      <c r="H3" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B4" t="s">
+        <v>447</v>
+      </c>
+      <c r="C4" t="s">
+        <v>448</v>
+      </c>
+      <c r="D4" t="s">
+        <v>454</v>
+      </c>
+      <c r="E4" t="s">
+        <v>447</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
+        <v>450</v>
+      </c>
+      <c r="H4" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>255</v>
+      </c>
+      <c r="B5" t="s">
+        <v>447</v>
+      </c>
+      <c r="C5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D5" t="s">
+        <v>455</v>
+      </c>
+      <c r="E5" t="s">
+        <v>447</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5" t="s">
+        <v>450</v>
+      </c>
+      <c r="H5" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>262</v>
+      </c>
+      <c r="B6" t="s">
+        <v>447</v>
+      </c>
+      <c r="C6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D6" t="s">
+        <v>456</v>
+      </c>
+      <c r="E6" t="s">
+        <v>447</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>450</v>
+      </c>
+      <c r="H6" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>269</v>
+      </c>
+      <c r="B7" t="s">
+        <v>447</v>
+      </c>
+      <c r="C7" t="s">
+        <v>448</v>
+      </c>
+      <c r="D7" t="s">
+        <v>457</v>
+      </c>
+      <c r="E7" t="s">
+        <v>447</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
+        <v>450</v>
+      </c>
+      <c r="H7" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>276</v>
+      </c>
+      <c r="B8" t="s">
+        <v>447</v>
+      </c>
+      <c r="C8" t="s">
+        <v>448</v>
+      </c>
+      <c r="D8" t="s">
+        <v>458</v>
+      </c>
+      <c r="E8" t="s">
+        <v>447</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8" t="s">
+        <v>450</v>
+      </c>
+      <c r="H8" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>283</v>
+      </c>
+      <c r="B9" t="s">
+        <v>447</v>
+      </c>
+      <c r="C9" t="s">
+        <v>448</v>
+      </c>
+      <c r="D9" t="s">
+        <v>459</v>
+      </c>
+      <c r="E9" t="s">
+        <v>447</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9" t="s">
+        <v>450</v>
+      </c>
+      <c r="H9" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>290</v>
+      </c>
+      <c r="B10" t="s">
+        <v>447</v>
+      </c>
+      <c r="C10" t="s">
+        <v>448</v>
+      </c>
+      <c r="D10" t="s">
+        <v>460</v>
+      </c>
+      <c r="E10" t="s">
+        <v>447</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10" t="s">
+        <v>450</v>
+      </c>
+      <c r="H10" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>297</v>
+      </c>
+      <c r="B11" t="s">
+        <v>447</v>
+      </c>
+      <c r="C11" t="s">
+        <v>448</v>
+      </c>
+      <c r="D11" t="s">
+        <v>461</v>
+      </c>
+      <c r="E11" t="s">
+        <v>447</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11" t="s">
+        <v>450</v>
+      </c>
+      <c r="H11" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>304</v>
+      </c>
+      <c r="B12" t="s">
+        <v>447</v>
+      </c>
+      <c r="C12" t="s">
+        <v>448</v>
+      </c>
+      <c r="D12" t="s">
+        <v>462</v>
+      </c>
+      <c r="E12" t="s">
+        <v>447</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12" t="s">
+        <v>450</v>
+      </c>
+      <c r="H12" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>311</v>
+      </c>
+      <c r="B13" t="s">
+        <v>447</v>
+      </c>
+      <c r="C13" t="s">
+        <v>448</v>
+      </c>
+      <c r="D13" t="s">
+        <v>463</v>
+      </c>
+      <c r="E13" t="s">
+        <v>447</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13" t="s">
+        <v>450</v>
+      </c>
+      <c r="H13" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>318</v>
+      </c>
+      <c r="B14" t="s">
+        <v>447</v>
+      </c>
+      <c r="C14" t="s">
+        <v>448</v>
+      </c>
+      <c r="D14" t="s">
+        <v>464</v>
+      </c>
+      <c r="E14" t="s">
+        <v>447</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14" t="s">
+        <v>450</v>
+      </c>
+      <c r="H14" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>325</v>
+      </c>
+      <c r="B15" t="s">
+        <v>447</v>
+      </c>
+      <c r="C15" t="s">
+        <v>448</v>
+      </c>
+      <c r="D15" t="s">
+        <v>465</v>
+      </c>
+      <c r="E15" t="s">
+        <v>447</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15" t="s">
+        <v>450</v>
+      </c>
+      <c r="H15" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>466</v>
+      </c>
+      <c r="B16" t="s">
+        <v>447</v>
+      </c>
+      <c r="C16" t="s">
+        <v>448</v>
+      </c>
+      <c r="D16" t="s">
+        <v>467</v>
+      </c>
+      <c r="E16" t="s">
+        <v>447</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16" t="s">
+        <v>450</v>
+      </c>
+      <c r="H16" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>468</v>
+      </c>
+      <c r="B17" t="s">
+        <v>447</v>
+      </c>
+      <c r="C17" t="s">
+        <v>448</v>
+      </c>
+      <c r="D17" t="s">
+        <v>469</v>
+      </c>
+      <c r="E17" t="s">
+        <v>447</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17" t="s">
+        <v>450</v>
+      </c>
+      <c r="H17" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>470</v>
+      </c>
+      <c r="B18" t="s">
+        <v>447</v>
+      </c>
+      <c r="C18" t="s">
+        <v>448</v>
+      </c>
+      <c r="D18" t="s">
+        <v>471</v>
+      </c>
+      <c r="E18" t="s">
+        <v>447</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18" t="s">
+        <v>450</v>
+      </c>
+      <c r="H18" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>405</v>
+      </c>
+      <c r="B19" t="s">
+        <v>447</v>
+      </c>
+      <c r="C19" t="s">
+        <v>448</v>
+      </c>
+      <c r="D19" t="s">
+        <v>472</v>
+      </c>
+      <c r="E19" t="s">
+        <v>447</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19" t="s">
+        <v>450</v>
+      </c>
+      <c r="H19" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>406</v>
+      </c>
+      <c r="B20" t="s">
+        <v>447</v>
+      </c>
+      <c r="C20" t="s">
+        <v>448</v>
+      </c>
+      <c r="D20" t="s">
+        <v>473</v>
+      </c>
+      <c r="E20" t="s">
+        <v>447</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20" t="s">
+        <v>450</v>
+      </c>
+      <c r="H20" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>474</v>
+      </c>
+      <c r="B21" t="s">
+        <v>447</v>
+      </c>
+      <c r="C21" t="s">
+        <v>448</v>
+      </c>
+      <c r="D21" t="s">
+        <v>475</v>
+      </c>
+      <c r="E21" t="s">
+        <v>447</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21" t="s">
+        <v>450</v>
+      </c>
+      <c r="H21" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>407</v>
+      </c>
+      <c r="B22" t="s">
+        <v>447</v>
+      </c>
+      <c r="C22" t="s">
+        <v>448</v>
+      </c>
+      <c r="D22" t="s">
+        <v>476</v>
+      </c>
+      <c r="E22" t="s">
+        <v>447</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22" t="s">
+        <v>450</v>
+      </c>
+      <c r="H22" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>409</v>
+      </c>
+      <c r="B23" t="s">
+        <v>447</v>
+      </c>
+      <c r="C23" t="s">
+        <v>448</v>
+      </c>
+      <c r="D23" t="s">
+        <v>477</v>
+      </c>
+      <c r="E23" t="s">
+        <v>447</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23" t="s">
+        <v>450</v>
+      </c>
+      <c r="H23" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>478</v>
+      </c>
+      <c r="B24" t="s">
+        <v>447</v>
+      </c>
+      <c r="C24" t="s">
+        <v>448</v>
+      </c>
+      <c r="D24" t="s">
+        <v>479</v>
+      </c>
+      <c r="E24" t="s">
+        <v>447</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24" t="s">
+        <v>450</v>
+      </c>
+      <c r="H24" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>480</v>
+      </c>
+      <c r="B25" t="s">
+        <v>447</v>
+      </c>
+      <c r="C25" t="s">
+        <v>448</v>
+      </c>
+      <c r="D25" t="s">
+        <v>481</v>
+      </c>
+      <c r="E25" t="s">
+        <v>447</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25" t="s">
+        <v>450</v>
+      </c>
+      <c r="H25" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>482</v>
+      </c>
+      <c r="B26" t="s">
+        <v>447</v>
+      </c>
+      <c r="C26" t="s">
+        <v>448</v>
+      </c>
+      <c r="D26" t="s">
+        <v>483</v>
+      </c>
+      <c r="E26" t="s">
+        <v>447</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26" t="s">
+        <v>450</v>
+      </c>
+      <c r="H26" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>484</v>
+      </c>
+      <c r="B27" t="s">
+        <v>447</v>
+      </c>
+      <c r="C27" t="s">
+        <v>448</v>
+      </c>
+      <c r="D27" t="s">
+        <v>485</v>
+      </c>
+      <c r="E27" t="s">
+        <v>447</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" t="s">
+        <v>450</v>
+      </c>
+      <c r="H27" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>486</v>
+      </c>
+      <c r="B28" t="s">
+        <v>447</v>
+      </c>
+      <c r="C28" t="s">
+        <v>448</v>
+      </c>
+      <c r="D28" t="s">
+        <v>487</v>
+      </c>
+      <c r="E28" t="s">
+        <v>447</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28" t="s">
+        <v>450</v>
+      </c>
+      <c r="H28" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>488</v>
+      </c>
+      <c r="B29" t="s">
+        <v>447</v>
+      </c>
+      <c r="C29" t="s">
+        <v>448</v>
+      </c>
+      <c r="D29" t="s">
+        <v>489</v>
+      </c>
+      <c r="E29" t="s">
+        <v>447</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29" t="s">
+        <v>450</v>
+      </c>
+      <c r="H29" t="s">
+        <v>451</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{085F676F-525D-4676-9613-88ED455FD340}">
+  <dimension ref="A2:D31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>508</v>
+      </c>
+      <c r="B2" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>446</v>
+      </c>
+      <c r="B3" s="93">
+        <v>362.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B4" s="93">
+        <v>362.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>241</v>
+      </c>
+      <c r="B5" s="93">
+        <v>361.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>248</v>
+      </c>
+      <c r="B6" s="93">
+        <v>362.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>255</v>
+      </c>
+      <c r="B7" s="93">
+        <v>362.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>262</v>
+      </c>
+      <c r="B8" s="93">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>269</v>
+      </c>
+      <c r="B9" s="93">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>276</v>
+      </c>
+      <c r="B10" s="93">
+        <v>772.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>283</v>
+      </c>
+      <c r="B11" s="93">
+        <v>629.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>290</v>
+      </c>
+      <c r="B12" s="96">
+        <v>903.7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>297</v>
+      </c>
+      <c r="B13" s="96">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>304</v>
+      </c>
+      <c r="B14" s="96">
+        <v>711.1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>311</v>
+      </c>
+      <c r="B15" s="96">
+        <v>622.20000000000005</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>318</v>
+      </c>
+      <c r="B16" s="96">
+        <v>790.4</v>
+      </c>
+      <c r="D16" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>325</v>
+      </c>
+      <c r="B17" s="96">
+        <v>697</v>
+      </c>
+      <c r="D17" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>466</v>
+      </c>
+      <c r="B18" s="96">
+        <v>714.4</v>
+      </c>
+      <c r="D18" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>468</v>
+      </c>
+      <c r="B19" s="96">
+        <v>636.9</v>
+      </c>
+      <c r="D19" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>470</v>
+      </c>
+      <c r="B20" s="96">
+        <v>990.1</v>
+      </c>
+      <c r="D20" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>405</v>
+      </c>
+      <c r="B21" s="96">
+        <v>840.1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>406</v>
+      </c>
+      <c r="B22" s="96">
+        <v>737</v>
+      </c>
+      <c r="D22" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>474</v>
+      </c>
+      <c r="B23" s="96">
+        <v>545.79999999999995</v>
+      </c>
+      <c r="D23" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>407</v>
+      </c>
+      <c r="B24" s="99">
+        <v>885.6</v>
+      </c>
+      <c r="D24" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>409</v>
+      </c>
+      <c r="B25" s="99">
+        <v>741.4</v>
+      </c>
+      <c r="D25" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>478</v>
+      </c>
+      <c r="B26" s="99">
+        <v>642.70000000000005</v>
+      </c>
+      <c r="D26" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>480</v>
+      </c>
+      <c r="B27" s="99">
+        <v>598.1</v>
+      </c>
+      <c r="D27" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>482</v>
+      </c>
+      <c r="B28" s="99">
+        <v>1223.2</v>
+      </c>
+      <c r="D28" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>484</v>
+      </c>
+      <c r="B29" s="99">
+        <v>1083.0999999999999</v>
+      </c>
+      <c r="D29" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>486</v>
+      </c>
+      <c r="B30" s="99">
+        <v>1083.0999999999999</v>
+      </c>
+      <c r="D30" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>488</v>
+      </c>
+      <c r="B31" s="99">
+        <v>1081.0999999999999</v>
+      </c>
+      <c r="D31" t="s">
+        <v>507</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7729A820-E01A-4B4F-BEC5-72896FA52F21}">
   <dimension ref="A1:J31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -18850,14 +19967,14 @@
       <c r="B1">
         <v>25</v>
       </c>
-      <c r="D1" s="110" t="s">
+      <c r="D1" s="100" t="s">
         <v>490</v>
       </c>
-      <c r="E1" s="110">
+      <c r="E1" s="100">
         <v>50</v>
       </c>
-      <c r="F1" s="110"/>
-      <c r="G1" s="110"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
@@ -18866,16 +19983,16 @@
       <c r="B2" t="s">
         <v>330</v>
       </c>
-      <c r="D2" s="110" t="s">
+      <c r="D2" s="100" t="s">
         <v>412</v>
       </c>
-      <c r="E2" s="110" t="s">
+      <c r="E2" s="100" t="s">
         <v>413</v>
       </c>
-      <c r="F2" s="110" t="s">
+      <c r="F2" s="100" t="s">
         <v>414</v>
       </c>
-      <c r="G2" s="110" t="s">
+      <c r="G2" s="100" t="s">
         <v>415</v>
       </c>
       <c r="J2" t="s">
@@ -18889,16 +20006,16 @@
       <c r="B3" s="15">
         <v>191.3</v>
       </c>
-      <c r="D3" s="101" t="s">
+      <c r="D3" s="91" t="s">
         <v>416</v>
       </c>
-      <c r="E3" s="102" t="s">
+      <c r="E3" s="92" t="s">
         <v>417</v>
       </c>
-      <c r="F3" s="103">
+      <c r="F3" s="93">
         <v>362.4</v>
       </c>
-      <c r="G3" s="103">
+      <c r="G3" s="93">
         <v>362.4</v>
       </c>
       <c r="J3" t="s">
@@ -18912,16 +20029,16 @@
       <c r="B4" s="15">
         <v>190.3</v>
       </c>
-      <c r="D4" s="101" t="s">
+      <c r="D4" s="91" t="s">
         <v>418</v>
       </c>
-      <c r="E4" s="102" t="s">
+      <c r="E4" s="92" t="s">
         <v>417</v>
       </c>
-      <c r="F4" s="103">
+      <c r="F4" s="93">
         <v>362.4</v>
       </c>
-      <c r="G4" s="103">
+      <c r="G4" s="93">
         <v>362.4</v>
       </c>
       <c r="J4" t="s">
@@ -18935,16 +20052,16 @@
       <c r="B5" s="15">
         <v>190.3</v>
       </c>
-      <c r="D5" s="101" t="s">
+      <c r="D5" s="91" t="s">
         <v>419</v>
       </c>
-      <c r="E5" s="102" t="s">
+      <c r="E5" s="92" t="s">
         <v>417</v>
       </c>
-      <c r="F5" s="103">
+      <c r="F5" s="93">
         <v>361.4</v>
       </c>
-      <c r="G5" s="103">
+      <c r="G5" s="93">
         <v>361.4</v>
       </c>
       <c r="J5" t="s">
@@ -18958,16 +20075,16 @@
       <c r="B6" s="15">
         <v>186.9</v>
       </c>
-      <c r="D6" s="101" t="s">
+      <c r="D6" s="91" t="s">
         <v>420</v>
       </c>
-      <c r="E6" s="102" t="s">
+      <c r="E6" s="92" t="s">
         <v>417</v>
       </c>
-      <c r="F6" s="103">
+      <c r="F6" s="93">
         <v>362.4</v>
       </c>
-      <c r="G6" s="103">
+      <c r="G6" s="93">
         <v>362.4</v>
       </c>
       <c r="J6" t="s">
@@ -18981,16 +20098,16 @@
       <c r="B7" s="15">
         <v>191.3</v>
       </c>
-      <c r="D7" s="101" t="s">
+      <c r="D7" s="91" t="s">
         <v>421</v>
       </c>
-      <c r="E7" s="102" t="s">
+      <c r="E7" s="92" t="s">
         <v>417</v>
       </c>
-      <c r="F7" s="103">
+      <c r="F7" s="93">
         <v>362.4</v>
       </c>
-      <c r="G7" s="103">
+      <c r="G7" s="93">
         <v>362.4</v>
       </c>
       <c r="J7" t="s">
@@ -19004,16 +20121,16 @@
       <c r="B8" s="15">
         <v>191.3</v>
       </c>
-      <c r="D8" s="101" t="s">
+      <c r="D8" s="91" t="s">
         <v>422</v>
       </c>
-      <c r="E8" s="102" t="s">
+      <c r="E8" s="92" t="s">
         <v>417</v>
       </c>
-      <c r="F8" s="103">
+      <c r="F8" s="93">
         <v>1044</v>
       </c>
-      <c r="G8" s="103">
+      <c r="G8" s="93">
         <v>1043.3</v>
       </c>
       <c r="J8" t="s">
@@ -19027,16 +20144,16 @@
       <c r="B9" s="15">
         <v>191.3</v>
       </c>
-      <c r="D9" s="101" t="s">
+      <c r="D9" s="91" t="s">
         <v>423</v>
       </c>
-      <c r="E9" s="102" t="s">
+      <c r="E9" s="92" t="s">
         <v>417</v>
       </c>
-      <c r="F9" s="103">
+      <c r="F9" s="93">
         <v>909</v>
       </c>
-      <c r="G9" s="103">
+      <c r="G9" s="93">
         <v>909</v>
       </c>
       <c r="J9" t="s">
@@ -19050,16 +20167,16 @@
       <c r="B10" s="18">
         <v>191.3</v>
       </c>
-      <c r="D10" s="101" t="s">
+      <c r="D10" s="91" t="s">
         <v>424</v>
       </c>
-      <c r="E10" s="102" t="s">
+      <c r="E10" s="92" t="s">
         <v>417</v>
       </c>
-      <c r="F10" s="103">
+      <c r="F10" s="93">
         <v>772.9</v>
       </c>
-      <c r="G10" s="103">
+      <c r="G10" s="93">
         <v>769.2</v>
       </c>
       <c r="J10" t="s">
@@ -19073,16 +20190,16 @@
       <c r="B11" s="18">
         <v>191.3</v>
       </c>
-      <c r="D11" s="101" t="s">
+      <c r="D11" s="91" t="s">
         <v>425</v>
       </c>
-      <c r="E11" s="102" t="s">
+      <c r="E11" s="92" t="s">
         <v>417</v>
       </c>
-      <c r="F11" s="103">
+      <c r="F11" s="93">
         <v>629.4</v>
       </c>
-      <c r="G11" s="103">
+      <c r="G11" s="93">
         <v>619.1</v>
       </c>
       <c r="J11" t="s">
@@ -19096,16 +20213,16 @@
       <c r="B12" s="19">
         <v>617.1</v>
       </c>
-      <c r="D12" s="104" t="s">
+      <c r="D12" s="94" t="s">
         <v>426</v>
       </c>
-      <c r="E12" s="105" t="s">
+      <c r="E12" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F12" s="106">
+      <c r="F12" s="96">
         <v>903.7</v>
       </c>
-      <c r="G12" s="106">
+      <c r="G12" s="96">
         <v>892.1</v>
       </c>
       <c r="J12" t="s">
@@ -19119,16 +20236,16 @@
       <c r="B13" s="18">
         <v>547.1</v>
       </c>
-      <c r="D13" s="104" t="s">
+      <c r="D13" s="94" t="s">
         <v>427</v>
       </c>
-      <c r="E13" s="105" t="s">
+      <c r="E13" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F13" s="106">
+      <c r="F13" s="96">
         <v>793</v>
       </c>
-      <c r="G13" s="106">
+      <c r="G13" s="96">
         <v>791.3</v>
       </c>
       <c r="J13" t="s">
@@ -19142,16 +20259,16 @@
       <c r="B14" s="18">
         <v>454.6</v>
       </c>
-      <c r="D14" s="104" t="s">
+      <c r="D14" s="94" t="s">
         <v>428</v>
       </c>
-      <c r="E14" s="105" t="s">
+      <c r="E14" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F14" s="106">
+      <c r="F14" s="96">
         <v>711.1</v>
       </c>
-      <c r="G14" s="106">
+      <c r="G14" s="96">
         <v>707.2</v>
       </c>
       <c r="J14" t="s">
@@ -19165,16 +20282,16 @@
       <c r="B15" s="18">
         <v>416.9</v>
       </c>
-      <c r="D15" s="104" t="s">
+      <c r="D15" s="94" t="s">
         <v>429</v>
       </c>
-      <c r="E15" s="105" t="s">
+      <c r="E15" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F15" s="106">
+      <c r="F15" s="96">
         <v>622.20000000000005</v>
       </c>
-      <c r="G15" s="106">
+      <c r="G15" s="96">
         <v>594.70000000000005</v>
       </c>
       <c r="J15" t="s">
@@ -19188,16 +20305,16 @@
       <c r="B16" s="18">
         <v>530.5</v>
       </c>
-      <c r="D16" s="104" t="s">
+      <c r="D16" s="94" t="s">
         <v>430</v>
       </c>
-      <c r="E16" s="105" t="s">
+      <c r="E16" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F16" s="106">
+      <c r="F16" s="96">
         <v>790.4</v>
       </c>
-      <c r="G16" s="106">
+      <c r="G16" s="96">
         <v>775.3</v>
       </c>
       <c r="J16" t="s">
@@ -19211,16 +20328,16 @@
       <c r="B17" s="18">
         <v>465.4</v>
       </c>
-      <c r="D17" s="104" t="s">
+      <c r="D17" s="94" t="s">
         <v>431</v>
       </c>
-      <c r="E17" s="105" t="s">
+      <c r="E17" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F17" s="106">
+      <c r="F17" s="96">
         <v>697</v>
       </c>
-      <c r="G17" s="106">
+      <c r="G17" s="96">
         <v>695.1</v>
       </c>
       <c r="J17" t="s">
@@ -19234,16 +20351,16 @@
       <c r="B18" s="18">
         <v>424.3</v>
       </c>
-      <c r="D18" s="104" t="s">
+      <c r="D18" s="94" t="s">
         <v>432</v>
       </c>
-      <c r="E18" s="105" t="s">
+      <c r="E18" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F18" s="106">
+      <c r="F18" s="96">
         <v>714.4</v>
       </c>
-      <c r="G18" s="106">
+      <c r="G18" s="96">
         <v>696.3</v>
       </c>
       <c r="J18" t="s">
@@ -19257,16 +20374,16 @@
       <c r="B19" s="18">
         <v>397.3</v>
       </c>
-      <c r="D19" s="104" t="s">
+      <c r="D19" s="94" t="s">
         <v>433</v>
       </c>
-      <c r="E19" s="105" t="s">
+      <c r="E19" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F19" s="106">
+      <c r="F19" s="96">
         <v>636.9</v>
       </c>
-      <c r="G19" s="106">
+      <c r="G19" s="96">
         <v>614.79999999999995</v>
       </c>
       <c r="J19" t="s">
@@ -19280,16 +20397,16 @@
       <c r="B20" s="18">
         <v>441.3</v>
       </c>
-      <c r="D20" s="104" t="s">
+      <c r="D20" s="94" t="s">
         <v>434</v>
       </c>
-      <c r="E20" s="105" t="s">
+      <c r="E20" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F20" s="106">
+      <c r="F20" s="96">
         <v>990.1</v>
       </c>
-      <c r="G20" s="106">
+      <c r="G20" s="96">
         <v>850</v>
       </c>
       <c r="J20" t="s">
@@ -19303,16 +20420,16 @@
       <c r="B21" s="18">
         <v>444.1</v>
       </c>
-      <c r="D21" s="104" t="s">
+      <c r="D21" s="94" t="s">
         <v>435</v>
       </c>
-      <c r="E21" s="105" t="s">
+      <c r="E21" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F21" s="106">
+      <c r="F21" s="96">
         <v>840.1</v>
       </c>
-      <c r="G21" s="106">
+      <c r="G21" s="96">
         <v>721.8</v>
       </c>
       <c r="J21" t="s">
@@ -19326,16 +20443,16 @@
       <c r="B22" s="18">
         <v>428.8</v>
       </c>
-      <c r="D22" s="104" t="s">
+      <c r="D22" s="94" t="s">
         <v>436</v>
       </c>
-      <c r="E22" s="105" t="s">
+      <c r="E22" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F22" s="106">
+      <c r="F22" s="96">
         <v>737</v>
       </c>
-      <c r="G22" s="106">
+      <c r="G22" s="96">
         <v>645.20000000000005</v>
       </c>
       <c r="J22" t="s">
@@ -19349,16 +20466,16 @@
       <c r="B23" s="20">
         <v>393</v>
       </c>
-      <c r="D23" s="104" t="s">
+      <c r="D23" s="94" t="s">
         <v>437</v>
       </c>
-      <c r="E23" s="105" t="s">
+      <c r="E23" s="95" t="s">
         <v>403</v>
       </c>
-      <c r="F23" s="106">
+      <c r="F23" s="96">
         <v>545.79999999999995</v>
       </c>
-      <c r="G23" s="106">
+      <c r="G23" s="96">
         <v>545.79999999999995</v>
       </c>
       <c r="J23" t="s">
@@ -19372,16 +20489,16 @@
       <c r="B24" s="18">
         <v>461.1</v>
       </c>
-      <c r="D24" s="107" t="s">
+      <c r="D24" s="97" t="s">
         <v>438</v>
       </c>
-      <c r="E24" s="108" t="s">
+      <c r="E24" s="98" t="s">
         <v>408</v>
       </c>
-      <c r="F24" s="109">
+      <c r="F24" s="99">
         <v>885.6</v>
       </c>
-      <c r="G24" s="109">
+      <c r="G24" s="99">
         <v>761.5</v>
       </c>
       <c r="J24" t="s">
@@ -19395,16 +20512,16 @@
       <c r="B25" s="18">
         <v>351.8</v>
       </c>
-      <c r="D25" s="107" t="s">
+      <c r="D25" s="97" t="s">
         <v>439</v>
       </c>
-      <c r="E25" s="108" t="s">
+      <c r="E25" s="98" t="s">
         <v>408</v>
       </c>
-      <c r="F25" s="109">
+      <c r="F25" s="99">
         <v>741.4</v>
       </c>
-      <c r="G25" s="109">
+      <c r="G25" s="99">
         <v>664.4</v>
       </c>
       <c r="J25" t="s">
@@ -19418,16 +20535,16 @@
       <c r="B26" s="18">
         <v>332.8</v>
       </c>
-      <c r="D26" s="107" t="s">
+      <c r="D26" s="97" t="s">
         <v>440</v>
       </c>
-      <c r="E26" s="108" t="s">
+      <c r="E26" s="98" t="s">
         <v>408</v>
       </c>
-      <c r="F26" s="109">
+      <c r="F26" s="99">
         <v>642.70000000000005</v>
       </c>
-      <c r="G26" s="109">
+      <c r="G26" s="99">
         <v>603.5</v>
       </c>
       <c r="J26" t="s">
@@ -19441,16 +20558,16 @@
       <c r="B27" s="18">
         <v>306.60000000000002</v>
       </c>
-      <c r="D27" s="107" t="s">
+      <c r="D27" s="97" t="s">
         <v>441</v>
       </c>
-      <c r="E27" s="108" t="s">
+      <c r="E27" s="98" t="s">
         <v>408</v>
       </c>
-      <c r="F27" s="109">
+      <c r="F27" s="99">
         <v>598.1</v>
       </c>
-      <c r="G27" s="109">
+      <c r="G27" s="99">
         <v>541.1</v>
       </c>
       <c r="J27" t="s">
@@ -19464,16 +20581,16 @@
       <c r="B28" s="18">
         <v>411.3</v>
       </c>
-      <c r="D28" s="107" t="s">
+      <c r="D28" s="97" t="s">
         <v>442</v>
       </c>
-      <c r="E28" s="108" t="s">
+      <c r="E28" s="98" t="s">
         <v>408</v>
       </c>
-      <c r="F28" s="109">
+      <c r="F28" s="99">
         <v>1223.2</v>
       </c>
-      <c r="G28" s="109">
+      <c r="G28" s="99">
         <v>1164.4000000000001</v>
       </c>
       <c r="J28" t="s">
@@ -19487,16 +20604,16 @@
       <c r="B29" s="18">
         <v>345.5</v>
       </c>
-      <c r="D29" s="107" t="s">
+      <c r="D29" s="97" t="s">
         <v>443</v>
       </c>
-      <c r="E29" s="108" t="s">
+      <c r="E29" s="98" t="s">
         <v>408</v>
       </c>
-      <c r="F29" s="109">
+      <c r="F29" s="99">
         <v>1083.0999999999999</v>
       </c>
-      <c r="G29" s="109">
+      <c r="G29" s="99">
         <v>1041.2</v>
       </c>
       <c r="J29" t="s">
@@ -19510,16 +20627,16 @@
       <c r="B30" s="18">
         <v>298.3</v>
       </c>
-      <c r="D30" s="107" t="s">
+      <c r="D30" s="97" t="s">
         <v>444</v>
       </c>
-      <c r="E30" s="108" t="s">
+      <c r="E30" s="98" t="s">
         <v>408</v>
       </c>
-      <c r="F30" s="109">
+      <c r="F30" s="99">
         <v>1083.0999999999999</v>
       </c>
-      <c r="G30" s="109">
+      <c r="G30" s="99">
         <v>1041.2</v>
       </c>
       <c r="J30" t="s">
@@ -19533,784 +20650,20 @@
       <c r="B31" s="15">
         <v>294.5</v>
       </c>
-      <c r="D31" s="107" t="s">
+      <c r="D31" s="97" t="s">
         <v>445</v>
       </c>
-      <c r="E31" s="108" t="s">
+      <c r="E31" s="98" t="s">
         <v>408</v>
       </c>
-      <c r="F31" s="109">
+      <c r="F31" s="99">
         <v>1081.0999999999999</v>
       </c>
-      <c r="G31" s="109">
+      <c r="G31" s="99">
         <v>1001.2</v>
       </c>
       <c r="J31" t="s">
         <v>489</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6381B92-E053-4233-81A5-0B655C210782}">
-  <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>446</v>
-      </c>
-      <c r="B1" t="s">
-        <v>447</v>
-      </c>
-      <c r="C1" t="s">
-        <v>448</v>
-      </c>
-      <c r="D1" t="s">
-        <v>449</v>
-      </c>
-      <c r="E1" t="s">
-        <v>447</v>
-      </c>
-      <c r="F1">
-        <v>0</v>
-      </c>
-      <c r="G1" t="s">
-        <v>450</v>
-      </c>
-      <c r="H1" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>234</v>
-      </c>
-      <c r="B2" t="s">
-        <v>447</v>
-      </c>
-      <c r="C2" t="s">
-        <v>448</v>
-      </c>
-      <c r="D2" t="s">
-        <v>452</v>
-      </c>
-      <c r="E2" t="s">
-        <v>447</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2" t="s">
-        <v>450</v>
-      </c>
-      <c r="H2" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>241</v>
-      </c>
-      <c r="B3" t="s">
-        <v>447</v>
-      </c>
-      <c r="C3" t="s">
-        <v>448</v>
-      </c>
-      <c r="D3" t="s">
-        <v>453</v>
-      </c>
-      <c r="E3" t="s">
-        <v>447</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3" t="s">
-        <v>450</v>
-      </c>
-      <c r="H3" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>248</v>
-      </c>
-      <c r="B4" t="s">
-        <v>447</v>
-      </c>
-      <c r="C4" t="s">
-        <v>448</v>
-      </c>
-      <c r="D4" t="s">
-        <v>454</v>
-      </c>
-      <c r="E4" t="s">
-        <v>447</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4" t="s">
-        <v>450</v>
-      </c>
-      <c r="H4" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>255</v>
-      </c>
-      <c r="B5" t="s">
-        <v>447</v>
-      </c>
-      <c r="C5" t="s">
-        <v>448</v>
-      </c>
-      <c r="D5" t="s">
-        <v>455</v>
-      </c>
-      <c r="E5" t="s">
-        <v>447</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5" t="s">
-        <v>450</v>
-      </c>
-      <c r="H5" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>262</v>
-      </c>
-      <c r="B6" t="s">
-        <v>447</v>
-      </c>
-      <c r="C6" t="s">
-        <v>448</v>
-      </c>
-      <c r="D6" t="s">
-        <v>456</v>
-      </c>
-      <c r="E6" t="s">
-        <v>447</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6" t="s">
-        <v>450</v>
-      </c>
-      <c r="H6" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>269</v>
-      </c>
-      <c r="B7" t="s">
-        <v>447</v>
-      </c>
-      <c r="C7" t="s">
-        <v>448</v>
-      </c>
-      <c r="D7" t="s">
-        <v>457</v>
-      </c>
-      <c r="E7" t="s">
-        <v>447</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7" t="s">
-        <v>450</v>
-      </c>
-      <c r="H7" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>276</v>
-      </c>
-      <c r="B8" t="s">
-        <v>447</v>
-      </c>
-      <c r="C8" t="s">
-        <v>448</v>
-      </c>
-      <c r="D8" t="s">
-        <v>458</v>
-      </c>
-      <c r="E8" t="s">
-        <v>447</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8" t="s">
-        <v>450</v>
-      </c>
-      <c r="H8" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>283</v>
-      </c>
-      <c r="B9" t="s">
-        <v>447</v>
-      </c>
-      <c r="C9" t="s">
-        <v>448</v>
-      </c>
-      <c r="D9" t="s">
-        <v>459</v>
-      </c>
-      <c r="E9" t="s">
-        <v>447</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9" t="s">
-        <v>450</v>
-      </c>
-      <c r="H9" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>290</v>
-      </c>
-      <c r="B10" t="s">
-        <v>447</v>
-      </c>
-      <c r="C10" t="s">
-        <v>448</v>
-      </c>
-      <c r="D10" t="s">
-        <v>460</v>
-      </c>
-      <c r="E10" t="s">
-        <v>447</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10" t="s">
-        <v>450</v>
-      </c>
-      <c r="H10" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>297</v>
-      </c>
-      <c r="B11" t="s">
-        <v>447</v>
-      </c>
-      <c r="C11" t="s">
-        <v>448</v>
-      </c>
-      <c r="D11" t="s">
-        <v>461</v>
-      </c>
-      <c r="E11" t="s">
-        <v>447</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11" t="s">
-        <v>450</v>
-      </c>
-      <c r="H11" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>304</v>
-      </c>
-      <c r="B12" t="s">
-        <v>447</v>
-      </c>
-      <c r="C12" t="s">
-        <v>448</v>
-      </c>
-      <c r="D12" t="s">
-        <v>462</v>
-      </c>
-      <c r="E12" t="s">
-        <v>447</v>
-      </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="G12" t="s">
-        <v>450</v>
-      </c>
-      <c r="H12" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>311</v>
-      </c>
-      <c r="B13" t="s">
-        <v>447</v>
-      </c>
-      <c r="C13" t="s">
-        <v>448</v>
-      </c>
-      <c r="D13" t="s">
-        <v>463</v>
-      </c>
-      <c r="E13" t="s">
-        <v>447</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13" t="s">
-        <v>450</v>
-      </c>
-      <c r="H13" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>318</v>
-      </c>
-      <c r="B14" t="s">
-        <v>447</v>
-      </c>
-      <c r="C14" t="s">
-        <v>448</v>
-      </c>
-      <c r="D14" t="s">
-        <v>464</v>
-      </c>
-      <c r="E14" t="s">
-        <v>447</v>
-      </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-      <c r="G14" t="s">
-        <v>450</v>
-      </c>
-      <c r="H14" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>325</v>
-      </c>
-      <c r="B15" t="s">
-        <v>447</v>
-      </c>
-      <c r="C15" t="s">
-        <v>448</v>
-      </c>
-      <c r="D15" t="s">
-        <v>465</v>
-      </c>
-      <c r="E15" t="s">
-        <v>447</v>
-      </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15" t="s">
-        <v>450</v>
-      </c>
-      <c r="H15" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>466</v>
-      </c>
-      <c r="B16" t="s">
-        <v>447</v>
-      </c>
-      <c r="C16" t="s">
-        <v>448</v>
-      </c>
-      <c r="D16" t="s">
-        <v>467</v>
-      </c>
-      <c r="E16" t="s">
-        <v>447</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-      <c r="G16" t="s">
-        <v>450</v>
-      </c>
-      <c r="H16" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>468</v>
-      </c>
-      <c r="B17" t="s">
-        <v>447</v>
-      </c>
-      <c r="C17" t="s">
-        <v>448</v>
-      </c>
-      <c r="D17" t="s">
-        <v>469</v>
-      </c>
-      <c r="E17" t="s">
-        <v>447</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-      <c r="G17" t="s">
-        <v>450</v>
-      </c>
-      <c r="H17" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>470</v>
-      </c>
-      <c r="B18" t="s">
-        <v>447</v>
-      </c>
-      <c r="C18" t="s">
-        <v>448</v>
-      </c>
-      <c r="D18" t="s">
-        <v>471</v>
-      </c>
-      <c r="E18" t="s">
-        <v>447</v>
-      </c>
-      <c r="F18">
-        <v>0</v>
-      </c>
-      <c r="G18" t="s">
-        <v>450</v>
-      </c>
-      <c r="H18" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>405</v>
-      </c>
-      <c r="B19" t="s">
-        <v>447</v>
-      </c>
-      <c r="C19" t="s">
-        <v>448</v>
-      </c>
-      <c r="D19" t="s">
-        <v>472</v>
-      </c>
-      <c r="E19" t="s">
-        <v>447</v>
-      </c>
-      <c r="F19">
-        <v>0</v>
-      </c>
-      <c r="G19" t="s">
-        <v>450</v>
-      </c>
-      <c r="H19" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>406</v>
-      </c>
-      <c r="B20" t="s">
-        <v>447</v>
-      </c>
-      <c r="C20" t="s">
-        <v>448</v>
-      </c>
-      <c r="D20" t="s">
-        <v>473</v>
-      </c>
-      <c r="E20" t="s">
-        <v>447</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-      <c r="G20" t="s">
-        <v>450</v>
-      </c>
-      <c r="H20" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>474</v>
-      </c>
-      <c r="B21" t="s">
-        <v>447</v>
-      </c>
-      <c r="C21" t="s">
-        <v>448</v>
-      </c>
-      <c r="D21" t="s">
-        <v>475</v>
-      </c>
-      <c r="E21" t="s">
-        <v>447</v>
-      </c>
-      <c r="F21">
-        <v>0</v>
-      </c>
-      <c r="G21" t="s">
-        <v>450</v>
-      </c>
-      <c r="H21" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>407</v>
-      </c>
-      <c r="B22" t="s">
-        <v>447</v>
-      </c>
-      <c r="C22" t="s">
-        <v>448</v>
-      </c>
-      <c r="D22" t="s">
-        <v>476</v>
-      </c>
-      <c r="E22" t="s">
-        <v>447</v>
-      </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-      <c r="G22" t="s">
-        <v>450</v>
-      </c>
-      <c r="H22" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>409</v>
-      </c>
-      <c r="B23" t="s">
-        <v>447</v>
-      </c>
-      <c r="C23" t="s">
-        <v>448</v>
-      </c>
-      <c r="D23" t="s">
-        <v>477</v>
-      </c>
-      <c r="E23" t="s">
-        <v>447</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-      <c r="G23" t="s">
-        <v>450</v>
-      </c>
-      <c r="H23" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>478</v>
-      </c>
-      <c r="B24" t="s">
-        <v>447</v>
-      </c>
-      <c r="C24" t="s">
-        <v>448</v>
-      </c>
-      <c r="D24" t="s">
-        <v>479</v>
-      </c>
-      <c r="E24" t="s">
-        <v>447</v>
-      </c>
-      <c r="F24">
-        <v>0</v>
-      </c>
-      <c r="G24" t="s">
-        <v>450</v>
-      </c>
-      <c r="H24" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>480</v>
-      </c>
-      <c r="B25" t="s">
-        <v>447</v>
-      </c>
-      <c r="C25" t="s">
-        <v>448</v>
-      </c>
-      <c r="D25" t="s">
-        <v>481</v>
-      </c>
-      <c r="E25" t="s">
-        <v>447</v>
-      </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
-      <c r="G25" t="s">
-        <v>450</v>
-      </c>
-      <c r="H25" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>482</v>
-      </c>
-      <c r="B26" t="s">
-        <v>447</v>
-      </c>
-      <c r="C26" t="s">
-        <v>448</v>
-      </c>
-      <c r="D26" t="s">
-        <v>483</v>
-      </c>
-      <c r="E26" t="s">
-        <v>447</v>
-      </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-      <c r="G26" t="s">
-        <v>450</v>
-      </c>
-      <c r="H26" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>484</v>
-      </c>
-      <c r="B27" t="s">
-        <v>447</v>
-      </c>
-      <c r="C27" t="s">
-        <v>448</v>
-      </c>
-      <c r="D27" t="s">
-        <v>485</v>
-      </c>
-      <c r="E27" t="s">
-        <v>447</v>
-      </c>
-      <c r="F27">
-        <v>0</v>
-      </c>
-      <c r="G27" t="s">
-        <v>450</v>
-      </c>
-      <c r="H27" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>486</v>
-      </c>
-      <c r="B28" t="s">
-        <v>447</v>
-      </c>
-      <c r="C28" t="s">
-        <v>448</v>
-      </c>
-      <c r="D28" t="s">
-        <v>487</v>
-      </c>
-      <c r="E28" t="s">
-        <v>447</v>
-      </c>
-      <c r="F28">
-        <v>0</v>
-      </c>
-      <c r="G28" t="s">
-        <v>450</v>
-      </c>
-      <c r="H28" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>488</v>
-      </c>
-      <c r="B29" t="s">
-        <v>447</v>
-      </c>
-      <c r="C29" t="s">
-        <v>448</v>
-      </c>
-      <c r="D29" t="s">
-        <v>489</v>
-      </c>
-      <c r="E29" t="s">
-        <v>447</v>
-      </c>
-      <c r="F29">
-        <v>0</v>
-      </c>
-      <c r="G29" t="s">
-        <v>450</v>
-      </c>
-      <c r="H29" t="s">
-        <v>451</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
voltei excel analise e agora pronto para multijanelas
</commit_message>
<xml_diff>
--- a/analisesFinais.xlsx
+++ b/analisesFinais.xlsx
@@ -8,19 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PolyanaSilva\Documents\BP_VRPTW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E50BC8C-A3EB-464C-B9BF-F50CC3A0E2BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE8B37C0-7467-4E47-9D0F-CEE8DF777829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="2" xr2:uid="{E7DF56F7-393C-4179-80B5-2006709A41FF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{E7DF56F7-393C-4179-80B5-2006709A41FF}"/>
   </bookViews>
   <sheets>
     <sheet name="PRICING25" sheetId="2" r:id="rId1"/>
     <sheet name="SM25" sheetId="3" r:id="rId2"/>
     <sheet name="Análise_25nósComSemEstabIntegGe" sheetId="5" r:id="rId3"/>
-    <sheet name="FO_CONHECIDA" sheetId="4" r:id="rId4"/>
+    <sheet name="Construtiva50" sheetId="6" r:id="rId4"/>
+    <sheet name="50SM20" sheetId="7" r:id="rId5"/>
+    <sheet name="FO_CONHECIDA" sheetId="4" r:id="rId6"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId5"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PRICING25!$A$1:$V$117</definedName>
   </definedNames>
@@ -48,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1170" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1514" uniqueCount="510">
   <si>
     <t>run_id</t>
   </si>
@@ -1284,6 +1283,300 @@
   </si>
   <si>
     <t xml:space="preserve">Análise feita para </t>
+  </si>
+  <si>
+    <t>Instancia</t>
+  </si>
+  <si>
+    <t>Familia</t>
+  </si>
+  <si>
+    <t>UB_lit</t>
+  </si>
+  <si>
+    <t>LB_lit</t>
+  </si>
+  <si>
+    <t>C101N</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>C102</t>
+  </si>
+  <si>
+    <t>C103</t>
+  </si>
+  <si>
+    <t>C104</t>
+  </si>
+  <si>
+    <t>C105</t>
+  </si>
+  <si>
+    <t>C106</t>
+  </si>
+  <si>
+    <t>C107</t>
+  </si>
+  <si>
+    <t>C108</t>
+  </si>
+  <si>
+    <t>C109</t>
+  </si>
+  <si>
+    <t>R101</t>
+  </si>
+  <si>
+    <t>R102</t>
+  </si>
+  <si>
+    <t>R103</t>
+  </si>
+  <si>
+    <t>R104</t>
+  </si>
+  <si>
+    <t>R105</t>
+  </si>
+  <si>
+    <t>R106</t>
+  </si>
+  <si>
+    <t>R107</t>
+  </si>
+  <si>
+    <t>R108</t>
+  </si>
+  <si>
+    <t>R109</t>
+  </si>
+  <si>
+    <t>R110</t>
+  </si>
+  <si>
+    <t>R111</t>
+  </si>
+  <si>
+    <t>R112</t>
+  </si>
+  <si>
+    <t>RC101</t>
+  </si>
+  <si>
+    <t>RC102</t>
+  </si>
+  <si>
+    <t>RC103</t>
+  </si>
+  <si>
+    <t>RC104</t>
+  </si>
+  <si>
+    <t>RC105</t>
+  </si>
+  <si>
+    <t>RC106</t>
+  </si>
+  <si>
+    <t>RC107</t>
+  </si>
+  <si>
+    <t>RC108</t>
+  </si>
+  <si>
+    <t>c101n</t>
+  </si>
+  <si>
+    <t>|</t>
+  </si>
+  <si>
+    <t>custo=</t>
+  </si>
+  <si>
+    <t>362.4</t>
+  </si>
+  <si>
+    <t>art</t>
+  </si>
+  <si>
+    <t>✓</t>
+  </si>
+  <si>
+    <t>376.4</t>
+  </si>
+  <si>
+    <t>410.4</t>
+  </si>
+  <si>
+    <t>402.1</t>
+  </si>
+  <si>
+    <t>373.5</t>
+  </si>
+  <si>
+    <t>365.4</t>
+  </si>
+  <si>
+    <t>365.2</t>
+  </si>
+  <si>
+    <t>431.3</t>
+  </si>
+  <si>
+    <t>391.1</t>
+  </si>
+  <si>
+    <t>1139.3</t>
+  </si>
+  <si>
+    <t>946.5</t>
+  </si>
+  <si>
+    <t>911.3</t>
+  </si>
+  <si>
+    <t>746.6</t>
+  </si>
+  <si>
+    <t>1016.8</t>
+  </si>
+  <si>
+    <t>888.7</t>
+  </si>
+  <si>
+    <t>r107</t>
+  </si>
+  <si>
+    <t>919.3</t>
+  </si>
+  <si>
+    <t>r108</t>
+  </si>
+  <si>
+    <t>763.8</t>
+  </si>
+  <si>
+    <t>r109</t>
+  </si>
+  <si>
+    <t>876.8</t>
+  </si>
+  <si>
+    <t>900.8</t>
+  </si>
+  <si>
+    <t>784.8</t>
+  </si>
+  <si>
+    <t>r112</t>
+  </si>
+  <si>
+    <t>734.3</t>
+  </si>
+  <si>
+    <t>914.6</t>
+  </si>
+  <si>
+    <t>885.3</t>
+  </si>
+  <si>
+    <t>rc103</t>
+  </si>
+  <si>
+    <t>768.3</t>
+  </si>
+  <si>
+    <t>rc104</t>
+  </si>
+  <si>
+    <t>584.1</t>
+  </si>
+  <si>
+    <t>rc105</t>
+  </si>
+  <si>
+    <t>940.2</t>
+  </si>
+  <si>
+    <t>rc106</t>
+  </si>
+  <si>
+    <t>776.3</t>
+  </si>
+  <si>
+    <t>rc107</t>
+  </si>
+  <si>
+    <t>774.8</t>
+  </si>
+  <si>
+    <t>rc108</t>
+  </si>
+  <si>
+    <t>654.1</t>
+  </si>
+  <si>
+    <t>nos</t>
+  </si>
+  <si>
+    <t>Construtiva 50</t>
+  </si>
+  <si>
+    <t>902.80</t>
+  </si>
+  <si>
+    <t>888.70</t>
+  </si>
+  <si>
+    <t>711.10</t>
+  </si>
+  <si>
+    <t>763.80</t>
+  </si>
+  <si>
+    <t>876.80</t>
+  </si>
+  <si>
+    <t>900.80</t>
+  </si>
+  <si>
+    <t>784.80</t>
+  </si>
+  <si>
+    <t>734.30</t>
+  </si>
+  <si>
+    <t>1034.50</t>
+  </si>
+  <si>
+    <t>737.80</t>
+  </si>
+  <si>
+    <t>768.30</t>
+  </si>
+  <si>
+    <t>545.80</t>
+  </si>
+  <si>
+    <t>883.30</t>
+  </si>
+  <si>
+    <t>770.00</t>
+  </si>
+  <si>
+    <t>721.90</t>
+  </si>
+  <si>
+    <t>638.40</t>
+  </si>
+  <si>
+    <t>Inst</t>
+  </si>
+  <si>
+    <t>FoConhecido</t>
   </si>
 </sst>
 </file>
@@ -1297,7 +1590,7 @@
     <numFmt numFmtId="167" formatCode="\+0.0%;\-0.0%;\-"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1404,8 +1697,19 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1520,8 +1824,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF375623"/>
+        <bgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF5EB"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF0FB"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBF4EB"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -1669,13 +1997,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1711,22 +2054,7 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1795,22 +2123,10 @@
     <xf numFmtId="167" fontId="10" fillId="13" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="13" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1937,11 +2253,68 @@
     <xf numFmtId="0" fontId="13" fillId="13" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="21" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="22" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="22" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="23" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="23" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -4134,259 +4507,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Análise_25nósComSemEstabIntegGe"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="53">
-          <cell r="C53" t="str">
-            <v>COM Estab + Geo</v>
-          </cell>
-          <cell r="D53" t="str">
-            <v>COM Estab + Int</v>
-          </cell>
-          <cell r="E53" t="str">
-            <v>SEM Estab + Geo</v>
-          </cell>
-          <cell r="F53" t="str">
-            <v>SEM Estab + Int</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="B54" t="str">
-            <v>C (9)</v>
-          </cell>
-          <cell r="C54">
-            <v>1</v>
-          </cell>
-          <cell r="D54">
-            <v>1</v>
-          </cell>
-          <cell r="E54">
-            <v>0.88888888888888895</v>
-          </cell>
-          <cell r="F54">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="B55" t="str">
-            <v>R (12)</v>
-          </cell>
-          <cell r="C55">
-            <v>0.83333333333333304</v>
-          </cell>
-          <cell r="D55">
-            <v>1</v>
-          </cell>
-          <cell r="E55">
-            <v>0.83333333333333304</v>
-          </cell>
-          <cell r="F55">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="56">
-          <cell r="B56" t="str">
-            <v>RC (8)</v>
-          </cell>
-          <cell r="C56">
-            <v>0.875</v>
-          </cell>
-          <cell r="D56">
-            <v>1</v>
-          </cell>
-          <cell r="E56">
-            <v>0.875</v>
-          </cell>
-          <cell r="F56">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="57">
-          <cell r="B57" t="str">
-            <v>Geral (29)</v>
-          </cell>
-          <cell r="C57">
-            <v>0.89655172413793105</v>
-          </cell>
-          <cell r="D57">
-            <v>1</v>
-          </cell>
-          <cell r="E57">
-            <v>0.86206896551724099</v>
-          </cell>
-          <cell r="F57">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="61">
-          <cell r="C61" t="str">
-            <v>COM Estab + Geo</v>
-          </cell>
-          <cell r="D61" t="str">
-            <v>COM Estab + Int</v>
-          </cell>
-          <cell r="E61" t="str">
-            <v>SEM Estab + Geo</v>
-          </cell>
-          <cell r="F61" t="str">
-            <v>SEM Estab + Int</v>
-          </cell>
-          <cell r="H61" t="str">
-            <v>COM Estab + Geo</v>
-          </cell>
-          <cell r="I61" t="str">
-            <v>COM Estab + Int</v>
-          </cell>
-          <cell r="J61" t="str">
-            <v>SEM Estab + Geo</v>
-          </cell>
-          <cell r="K61" t="str">
-            <v>SEM Estab + Int</v>
-          </cell>
-        </row>
-        <row r="62">
-          <cell r="B62" t="str">
-            <v>C (9)</v>
-          </cell>
-          <cell r="C62">
-            <v>134.222222222222</v>
-          </cell>
-          <cell r="D62">
-            <v>160.777777777778</v>
-          </cell>
-          <cell r="E62">
-            <v>196.666666666667</v>
-          </cell>
-          <cell r="F62">
-            <v>305</v>
-          </cell>
-          <cell r="G62" t="str">
-            <v>C (9)</v>
-          </cell>
-          <cell r="H62">
-            <v>327.555555555556</v>
-          </cell>
-          <cell r="I62">
-            <v>324.88888888888903</v>
-          </cell>
-          <cell r="J62">
-            <v>509.222222222222</v>
-          </cell>
-          <cell r="K62">
-            <v>640.11111111111097</v>
-          </cell>
-        </row>
-        <row r="63">
-          <cell r="B63" t="str">
-            <v>R (12)</v>
-          </cell>
-          <cell r="C63">
-            <v>111.333333333333</v>
-          </cell>
-          <cell r="D63">
-            <v>156.416666666667</v>
-          </cell>
-          <cell r="E63">
-            <v>177.166666666667</v>
-          </cell>
-          <cell r="F63">
-            <v>191.083333333333</v>
-          </cell>
-          <cell r="G63" t="str">
-            <v>R (12)</v>
-          </cell>
-          <cell r="H63">
-            <v>499.5</v>
-          </cell>
-          <cell r="I63">
-            <v>517.16666666666697</v>
-          </cell>
-          <cell r="J63">
-            <v>717.58333333333303</v>
-          </cell>
-          <cell r="K63">
-            <v>719.58333333333303</v>
-          </cell>
-        </row>
-        <row r="64">
-          <cell r="B64" t="str">
-            <v>RC (8)</v>
-          </cell>
-          <cell r="C64">
-            <v>34.125</v>
-          </cell>
-          <cell r="D64">
-            <v>32.625</v>
-          </cell>
-          <cell r="E64">
-            <v>83</v>
-          </cell>
-          <cell r="F64">
-            <v>49.5</v>
-          </cell>
-          <cell r="G64" t="str">
-            <v>RC (8)</v>
-          </cell>
-          <cell r="H64">
-            <v>173.875</v>
-          </cell>
-          <cell r="I64">
-            <v>91.625</v>
-          </cell>
-          <cell r="J64">
-            <v>285.375</v>
-          </cell>
-          <cell r="K64">
-            <v>143</v>
-          </cell>
-        </row>
-        <row r="65">
-          <cell r="B65" t="str">
-            <v>Geral (29)</v>
-          </cell>
-          <cell r="C65">
-            <v>97.137931034482804</v>
-          </cell>
-          <cell r="D65">
-            <v>123.620689655172</v>
-          </cell>
-          <cell r="E65">
-            <v>157.241379310345</v>
-          </cell>
-          <cell r="F65">
-            <v>187.37931034482801</v>
-          </cell>
-          <cell r="G65" t="str">
-            <v>Geral (29)</v>
-          </cell>
-          <cell r="H65">
-            <v>356.31034482758599</v>
-          </cell>
-          <cell r="I65">
-            <v>340.10344827586198</v>
-          </cell>
-          <cell r="J65">
-            <v>533.68965517241395</v>
-          </cell>
-          <cell r="K65">
-            <v>535.86206896551698</v>
-          </cell>
-        </row>
-      </sheetData>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
@@ -12968,8 +13088,10 @@
   <dimension ref="A1:X106"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.21875" style="3" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="12.88671875" customWidth="1"/>
@@ -13054,15 +13176,15 @@
       <c r="M2">
         <v>78.450450897216797</v>
       </c>
-      <c r="R2" s="21" t="s">
+      <c r="R2" s="101" t="s">
         <v>220</v>
       </c>
-      <c r="S2" s="22"/>
-      <c r="T2" s="22"/>
-      <c r="U2" s="22"/>
-      <c r="V2" s="22"/>
-      <c r="W2" s="22"/>
-      <c r="X2" s="22"/>
+      <c r="S2" s="102"/>
+      <c r="T2" s="102"/>
+      <c r="U2" s="102"/>
+      <c r="V2" s="102"/>
+      <c r="W2" s="102"/>
+      <c r="X2" s="102"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -13294,7 +13416,7 @@
       <c r="M6">
         <v>129.55700397491461</v>
       </c>
-      <c r="R6" s="100">
+      <c r="R6" s="90">
         <v>20</v>
       </c>
       <c r="S6" s="11">
@@ -17349,1402 +17471,1414 @@
   <dimension ref="B1:R81"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2" style="24" customWidth="1"/>
-    <col min="2" max="2" width="27" style="24" customWidth="1"/>
-    <col min="3" max="6" width="12" style="24" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" style="24" customWidth="1"/>
-    <col min="8" max="8" width="14" style="24" customWidth="1"/>
-    <col min="9" max="12" width="12" style="24" customWidth="1"/>
-    <col min="13" max="13" width="2" style="24" customWidth="1"/>
-    <col min="14" max="14" width="14" style="24" customWidth="1"/>
-    <col min="15" max="18" width="12" style="24" customWidth="1"/>
-    <col min="19" max="19" width="2" style="24" customWidth="1"/>
-    <col min="20" max="16384" width="8.6640625" style="24"/>
+    <col min="1" max="1" width="2" style="21" customWidth="1"/>
+    <col min="2" max="2" width="27" style="21" customWidth="1"/>
+    <col min="3" max="6" width="12" style="21" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" style="21" customWidth="1"/>
+    <col min="8" max="8" width="14" style="21" customWidth="1"/>
+    <col min="9" max="12" width="12" style="21" customWidth="1"/>
+    <col min="13" max="13" width="2" style="21" customWidth="1"/>
+    <col min="14" max="14" width="14" style="21" customWidth="1"/>
+    <col min="15" max="18" width="12" style="21" customWidth="1"/>
+    <col min="19" max="19" width="2" style="21" customWidth="1"/>
+    <col min="20" max="16384" width="8.6640625" style="21"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:18" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="106" t="s">
         <v>346</v>
       </c>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
+      <c r="E1" s="106"/>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+      <c r="I1" s="106"/>
+      <c r="J1" s="106"/>
+      <c r="K1" s="106"/>
+      <c r="L1" s="106"/>
+      <c r="M1" s="106"/>
+      <c r="N1" s="106"/>
+      <c r="O1" s="106"/>
+      <c r="P1" s="106"/>
+      <c r="Q1" s="106"/>
+      <c r="R1" s="106"/>
     </row>
     <row r="2" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="107" t="s">
         <v>347</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="25"/>
-      <c r="P2" s="25"/>
-      <c r="Q2" s="25"/>
-      <c r="R2" s="25"/>
+      <c r="C2" s="107"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="107"/>
+      <c r="F2" s="107"/>
+      <c r="G2" s="107"/>
+      <c r="H2" s="107"/>
+      <c r="I2" s="107"/>
+      <c r="J2" s="107"/>
+      <c r="K2" s="107"/>
+      <c r="L2" s="107"/>
+      <c r="M2" s="107"/>
+      <c r="N2" s="107"/>
+      <c r="O2" s="107"/>
+      <c r="P2" s="107"/>
+      <c r="Q2" s="107"/>
+      <c r="R2" s="107"/>
     </row>
     <row r="4" spans="2:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="104" t="s">
         <v>348</v>
       </c>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
+      <c r="C4" s="104"/>
+      <c r="D4" s="104"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="104"/>
+      <c r="H4" s="104"/>
+      <c r="I4" s="104"/>
+      <c r="J4" s="104"/>
+      <c r="K4" s="104"/>
+      <c r="L4" s="104"/>
     </row>
     <row r="5" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="22" t="s">
         <v>349</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="22" t="s">
         <v>350</v>
       </c>
-      <c r="D5" s="27" t="s">
+      <c r="D5" s="22" t="s">
         <v>351</v>
       </c>
-      <c r="E5" s="27" t="s">
+      <c r="E5" s="22" t="s">
         <v>352</v>
       </c>
-      <c r="F5" s="27" t="s">
+      <c r="F5" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="G5" s="27" t="s">
+      <c r="G5" s="22" t="s">
         <v>354</v>
       </c>
-      <c r="I5" s="28" t="s">
+      <c r="I5" s="23" t="s">
         <v>355</v>
       </c>
-      <c r="J5" s="28" t="s">
+      <c r="J5" s="23" t="s">
         <v>356</v>
       </c>
-      <c r="K5" s="28" t="s">
+      <c r="K5" s="23" t="s">
         <v>357</v>
       </c>
-      <c r="L5" s="28" t="s">
+      <c r="L5" s="23" t="s">
         <v>358</v>
       </c>
-      <c r="N5" s="29"/>
+      <c r="N5" s="24"/>
     </row>
     <row r="6" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="25" t="s">
         <v>359</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="26" t="s">
         <v>360</v>
       </c>
-      <c r="D6" s="32">
+      <c r="D6" s="27">
         <v>0.89655172413793105</v>
       </c>
-      <c r="E6" s="33">
+      <c r="E6" s="28">
         <v>97.137931034482804</v>
       </c>
-      <c r="F6" s="33">
+      <c r="F6" s="28">
         <v>356.31034482758599</v>
       </c>
-      <c r="G6" s="34">
+      <c r="G6" s="29">
         <v>2.64965517241379E-4</v>
       </c>
-      <c r="H6" s="35"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="36">
+      <c r="H6" s="30"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="31">
         <v>-0.21422594142259399</v>
       </c>
-      <c r="K6" s="37">
+      <c r="K6" s="32">
         <v>4.7652843962283302E-2</v>
       </c>
-      <c r="L6" s="31"/>
+      <c r="L6" s="26"/>
     </row>
     <row r="7" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="33" t="s">
         <v>361</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="34" t="s">
         <v>362</v>
       </c>
-      <c r="D7" s="40">
+      <c r="D7" s="35">
         <v>1</v>
       </c>
-      <c r="E7" s="41">
+      <c r="E7" s="36">
         <v>123.620689655172</v>
       </c>
-      <c r="F7" s="41">
+      <c r="F7" s="36">
         <v>340.10344827586198</v>
       </c>
-      <c r="G7" s="42">
-        <v>0</v>
-      </c>
-      <c r="H7" s="35"/>
-      <c r="I7" s="43" t="s">
+      <c r="G7" s="37">
+        <v>0</v>
+      </c>
+      <c r="H7" s="30"/>
+      <c r="I7" s="38" t="s">
         <v>363</v>
       </c>
-      <c r="J7" s="43" t="s">
+      <c r="J7" s="38" t="s">
         <v>364</v>
       </c>
-      <c r="K7" s="43" t="s">
+      <c r="K7" s="38" t="s">
         <v>364</v>
       </c>
-      <c r="L7" s="43" t="s">
+      <c r="L7" s="38" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="8" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="39" t="s">
         <v>366</v>
       </c>
-      <c r="C8" s="31" t="s">
+      <c r="C8" s="26" t="s">
         <v>367</v>
       </c>
-      <c r="D8" s="32">
+      <c r="D8" s="27">
         <v>0.86206896551724099</v>
       </c>
-      <c r="E8" s="33">
+      <c r="E8" s="28">
         <v>157.241379310345</v>
       </c>
-      <c r="F8" s="33">
+      <c r="F8" s="28">
         <v>533.68965517241395</v>
       </c>
-      <c r="G8" s="34">
+      <c r="G8" s="29">
         <v>3.6773571428571402E-3</v>
       </c>
-      <c r="H8" s="35"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="37">
+      <c r="H8" s="30"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="32">
         <v>0.27196652719665299</v>
       </c>
-      <c r="K8" s="37">
+      <c r="K8" s="32">
         <v>0.56919801277501803</v>
       </c>
-      <c r="L8" s="31"/>
+      <c r="L8" s="26"/>
     </row>
     <row r="9" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="45" t="s">
+      <c r="B9" s="40" t="s">
         <v>368</v>
       </c>
-      <c r="C9" s="46" t="s">
+      <c r="C9" s="41" t="s">
         <v>362</v>
       </c>
-      <c r="D9" s="47">
+      <c r="D9" s="42">
         <v>1</v>
       </c>
-      <c r="E9" s="48">
+      <c r="E9" s="43">
         <v>187.37931034482801</v>
       </c>
-      <c r="F9" s="48">
+      <c r="F9" s="43">
         <v>535.86206896551698</v>
       </c>
-      <c r="G9" s="49">
+      <c r="G9" s="44">
         <v>4.22431341581118E-5</v>
       </c>
-      <c r="H9" s="35"/>
-      <c r="I9" s="46"/>
-      <c r="J9" s="50">
+      <c r="H9" s="30"/>
+      <c r="I9" s="41"/>
+      <c r="J9" s="45">
         <v>0.51576011157601098</v>
       </c>
-      <c r="K9" s="50">
+      <c r="K9" s="45">
         <v>0.57558552164655796</v>
       </c>
-      <c r="L9" s="46"/>
+      <c r="L9" s="41"/>
     </row>
     <row r="11" spans="2:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="51" t="s">
+      <c r="B11" s="108" t="s">
         <v>369</v>
       </c>
-      <c r="C11" s="51"/>
-      <c r="D11" s="51"/>
-      <c r="E11" s="51"/>
-      <c r="F11" s="51"/>
-      <c r="G11" s="51"/>
-      <c r="H11" s="51"/>
-      <c r="I11" s="51"/>
-      <c r="J11" s="51"/>
-      <c r="K11" s="51"/>
-      <c r="L11" s="51"/>
+      <c r="C11" s="108"/>
+      <c r="D11" s="108"/>
+      <c r="E11" s="108"/>
+      <c r="F11" s="108"/>
+      <c r="G11" s="108"/>
+      <c r="H11" s="108"/>
+      <c r="I11" s="108"/>
+      <c r="J11" s="108"/>
+      <c r="K11" s="108"/>
+      <c r="L11" s="108"/>
     </row>
     <row r="12" spans="2:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="22" t="s">
         <v>370</v>
       </c>
-      <c r="C12" s="52" t="s">
+      <c r="C12" s="105" t="s">
         <v>371</v>
       </c>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="52"/>
-      <c r="H12" s="52"/>
-      <c r="I12" s="52"/>
-      <c r="J12" s="52"/>
-      <c r="K12" s="52"/>
-      <c r="L12" s="52"/>
+      <c r="D12" s="105"/>
+      <c r="E12" s="105"/>
+      <c r="F12" s="105"/>
+      <c r="G12" s="105"/>
+      <c r="H12" s="105"/>
+      <c r="I12" s="105"/>
+      <c r="J12" s="105"/>
+      <c r="K12" s="105"/>
+      <c r="L12" s="105"/>
     </row>
     <row r="13" spans="2:18" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="53" t="s">
+      <c r="B13" s="46" t="s">
         <v>372</v>
       </c>
-      <c r="C13" s="54" t="s">
+      <c r="C13" s="109" t="s">
         <v>373</v>
       </c>
-      <c r="D13" s="54"/>
-      <c r="E13" s="54"/>
-      <c r="F13" s="54"/>
-      <c r="G13" s="54"/>
-      <c r="H13" s="54"/>
-      <c r="I13" s="54"/>
-      <c r="J13" s="54"/>
-      <c r="K13" s="54"/>
-      <c r="L13" s="54"/>
+      <c r="D13" s="109"/>
+      <c r="E13" s="109"/>
+      <c r="F13" s="109"/>
+      <c r="G13" s="109"/>
+      <c r="H13" s="109"/>
+      <c r="I13" s="109"/>
+      <c r="J13" s="109"/>
+      <c r="K13" s="109"/>
+      <c r="L13" s="109"/>
     </row>
     <row r="14" spans="2:18" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="47" t="s">
         <v>374</v>
       </c>
-      <c r="C14" s="56" t="s">
+      <c r="C14" s="110" t="s">
         <v>375</v>
       </c>
-      <c r="D14" s="56"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56"/>
-      <c r="G14" s="56"/>
-      <c r="H14" s="56"/>
-      <c r="I14" s="56"/>
-      <c r="J14" s="56"/>
-      <c r="K14" s="56"/>
-      <c r="L14" s="56"/>
+      <c r="D14" s="110"/>
+      <c r="E14" s="110"/>
+      <c r="F14" s="110"/>
+      <c r="G14" s="110"/>
+      <c r="H14" s="110"/>
+      <c r="I14" s="110"/>
+      <c r="J14" s="110"/>
+      <c r="K14" s="110"/>
+      <c r="L14" s="110"/>
     </row>
     <row r="15" spans="2:18" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="53" t="s">
+      <c r="B15" s="46" t="s">
         <v>376</v>
       </c>
-      <c r="C15" s="54" t="s">
+      <c r="C15" s="109" t="s">
         <v>377</v>
       </c>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="54"/>
-      <c r="H15" s="54"/>
-      <c r="I15" s="54"/>
-      <c r="J15" s="54"/>
-      <c r="K15" s="54"/>
-      <c r="L15" s="54"/>
+      <c r="D15" s="109"/>
+      <c r="E15" s="109"/>
+      <c r="F15" s="109"/>
+      <c r="G15" s="109"/>
+      <c r="H15" s="109"/>
+      <c r="I15" s="109"/>
+      <c r="J15" s="109"/>
+      <c r="K15" s="109"/>
+      <c r="L15" s="109"/>
     </row>
     <row r="16" spans="2:18" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="55" t="s">
+      <c r="B16" s="47" t="s">
         <v>378</v>
       </c>
-      <c r="C16" s="56" t="s">
+      <c r="C16" s="110" t="s">
         <v>379</v>
       </c>
-      <c r="D16" s="56"/>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="56"/>
-      <c r="H16" s="56"/>
-      <c r="I16" s="56"/>
-      <c r="J16" s="56"/>
-      <c r="K16" s="56"/>
-      <c r="L16" s="56"/>
+      <c r="D16" s="110"/>
+      <c r="E16" s="110"/>
+      <c r="F16" s="110"/>
+      <c r="G16" s="110"/>
+      <c r="H16" s="110"/>
+      <c r="I16" s="110"/>
+      <c r="J16" s="110"/>
+      <c r="K16" s="110"/>
+      <c r="L16" s="110"/>
     </row>
     <row r="18" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="104" t="s">
         <v>380</v>
       </c>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="26"/>
-      <c r="M18" s="26"/>
-      <c r="N18" s="26"/>
-      <c r="O18" s="26"/>
-      <c r="P18" s="26"/>
-      <c r="Q18" s="26"/>
+      <c r="C18" s="104"/>
+      <c r="D18" s="104"/>
+      <c r="E18" s="104"/>
+      <c r="F18" s="104"/>
+      <c r="G18" s="104"/>
+      <c r="H18" s="104"/>
+      <c r="I18" s="104"/>
+      <c r="J18" s="104"/>
+      <c r="K18" s="104"/>
+      <c r="L18" s="104"/>
+      <c r="M18" s="104"/>
+      <c r="N18" s="104"/>
+      <c r="O18" s="104"/>
+      <c r="P18" s="104"/>
+      <c r="Q18" s="104"/>
     </row>
     <row r="19" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="22" t="s">
         <v>381</v>
       </c>
-      <c r="C19" s="27" t="s">
+      <c r="C19" s="22" t="s">
         <v>382</v>
       </c>
-      <c r="D19" s="57" t="s">
+      <c r="D19" s="48" t="s">
         <v>359</v>
       </c>
-      <c r="E19" s="58" t="s">
+      <c r="E19" s="49" t="s">
         <v>361</v>
       </c>
-      <c r="F19" s="59" t="s">
+      <c r="F19" s="50" t="s">
         <v>366</v>
       </c>
-      <c r="G19" s="60" t="s">
+      <c r="G19" s="51" t="s">
         <v>368</v>
       </c>
-      <c r="H19" s="28" t="s">
+      <c r="H19" s="23" t="s">
         <v>383</v>
       </c>
     </row>
     <row r="20" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="61" t="s">
+      <c r="B20" s="52" t="s">
         <v>384</v>
       </c>
-      <c r="C20" s="62" t="s">
+      <c r="C20" s="53" t="s">
         <v>385</v>
       </c>
-      <c r="D20" s="63">
+      <c r="D20" s="54">
         <v>1</v>
       </c>
-      <c r="E20" s="64">
+      <c r="E20" s="55">
         <v>1</v>
       </c>
-      <c r="F20" s="63">
+      <c r="F20" s="54">
         <v>0.88888888888888895</v>
       </c>
-      <c r="G20" s="63">
+      <c r="G20" s="54">
         <v>1</v>
       </c>
-      <c r="H20" s="57" t="s">
+      <c r="H20" s="48" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="21" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="65"/>
-      <c r="C21" s="66" t="s">
+      <c r="B21" s="56"/>
+      <c r="C21" s="57" t="s">
         <v>387</v>
       </c>
-      <c r="D21" s="67">
+      <c r="D21" s="58">
         <v>134.222222222222</v>
       </c>
-      <c r="E21" s="68">
+      <c r="E21" s="59">
         <v>160.777777777778</v>
       </c>
-      <c r="F21" s="67">
+      <c r="F21" s="58">
         <v>196.666666666667</v>
       </c>
-      <c r="G21" s="67">
+      <c r="G21" s="58">
         <v>305</v>
       </c>
-      <c r="H21" s="57" t="s">
+      <c r="H21" s="48" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="22" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="65"/>
-      <c r="C22" s="62" t="s">
+      <c r="B22" s="56"/>
+      <c r="C22" s="53" t="s">
         <v>388</v>
       </c>
-      <c r="D22" s="69">
+      <c r="D22" s="60">
         <v>327.555555555556</v>
       </c>
-      <c r="E22" s="68">
+      <c r="E22" s="59">
         <v>324.88888888888903</v>
       </c>
-      <c r="F22" s="69">
+      <c r="F22" s="60">
         <v>509.222222222222</v>
       </c>
-      <c r="G22" s="69">
+      <c r="G22" s="60">
         <v>640.11111111111097</v>
       </c>
-      <c r="H22" s="58" t="s">
+      <c r="H22" s="49" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="23" spans="2:17" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="70"/>
-      <c r="C23" s="70"/>
-      <c r="D23" s="70"/>
-      <c r="E23" s="70"/>
-      <c r="F23" s="70"/>
-      <c r="G23" s="70"/>
-      <c r="H23" s="70"/>
+      <c r="B23" s="61"/>
+      <c r="C23" s="61"/>
+      <c r="D23" s="61"/>
+      <c r="E23" s="61"/>
+      <c r="F23" s="61"/>
+      <c r="G23" s="61"/>
+      <c r="H23" s="61"/>
     </row>
     <row r="24" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="71" t="s">
+      <c r="B24" s="62" t="s">
         <v>390</v>
       </c>
-      <c r="C24" s="72" t="s">
+      <c r="C24" s="63" t="s">
         <v>385</v>
       </c>
-      <c r="D24" s="73">
+      <c r="D24" s="64">
         <v>0.83333333333333304</v>
       </c>
-      <c r="E24" s="64">
+      <c r="E24" s="55">
         <v>1</v>
       </c>
-      <c r="F24" s="73">
+      <c r="F24" s="64">
         <v>0.83333333333333304</v>
       </c>
-      <c r="G24" s="73">
+      <c r="G24" s="64">
         <v>1</v>
       </c>
-      <c r="H24" s="58" t="s">
+      <c r="H24" s="49" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="25" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="74"/>
-      <c r="C25" s="66" t="s">
+      <c r="B25" s="65"/>
+      <c r="C25" s="57" t="s">
         <v>387</v>
       </c>
-      <c r="D25" s="67">
+      <c r="D25" s="58">
         <v>111.333333333333</v>
       </c>
-      <c r="E25" s="68">
+      <c r="E25" s="59">
         <v>156.416666666667</v>
       </c>
-      <c r="F25" s="67">
+      <c r="F25" s="58">
         <v>177.166666666667</v>
       </c>
-      <c r="G25" s="67">
+      <c r="G25" s="58">
         <v>191.083333333333</v>
       </c>
-      <c r="H25" s="57" t="s">
+      <c r="H25" s="48" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="26" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="74"/>
-      <c r="C26" s="72" t="s">
+      <c r="B26" s="65"/>
+      <c r="C26" s="63" t="s">
         <v>388</v>
       </c>
-      <c r="D26" s="75">
+      <c r="D26" s="66">
         <v>499.5</v>
       </c>
-      <c r="E26" s="68">
+      <c r="E26" s="59">
         <v>517.16666666666697</v>
       </c>
-      <c r="F26" s="75">
+      <c r="F26" s="66">
         <v>717.58333333333303</v>
       </c>
-      <c r="G26" s="75">
+      <c r="G26" s="66">
         <v>719.58333333333303</v>
       </c>
-      <c r="H26" s="57" t="s">
+      <c r="H26" s="48" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="27" spans="2:17" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="70"/>
-      <c r="C27" s="70"/>
-      <c r="D27" s="70"/>
-      <c r="E27" s="70"/>
-      <c r="F27" s="70"/>
-      <c r="G27" s="70"/>
-      <c r="H27" s="70"/>
+      <c r="B27" s="61"/>
+      <c r="C27" s="61"/>
+      <c r="D27" s="61"/>
+      <c r="E27" s="61"/>
+      <c r="F27" s="61"/>
+      <c r="G27" s="61"/>
+      <c r="H27" s="61"/>
     </row>
     <row r="28" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="76" t="s">
+      <c r="B28" s="67" t="s">
         <v>391</v>
       </c>
-      <c r="C28" s="77" t="s">
+      <c r="C28" s="68" t="s">
         <v>385</v>
       </c>
-      <c r="D28" s="78">
+      <c r="D28" s="69">
         <v>0.875</v>
       </c>
-      <c r="E28" s="64">
+      <c r="E28" s="55">
         <v>1</v>
       </c>
-      <c r="F28" s="78">
+      <c r="F28" s="69">
         <v>0.875</v>
       </c>
-      <c r="G28" s="78">
+      <c r="G28" s="69">
         <v>1</v>
       </c>
-      <c r="H28" s="58" t="s">
+      <c r="H28" s="49" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="29" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="79"/>
-      <c r="C29" s="66" t="s">
+      <c r="B29" s="70"/>
+      <c r="C29" s="57" t="s">
         <v>387</v>
       </c>
-      <c r="D29" s="67">
+      <c r="D29" s="58">
         <v>34.125</v>
       </c>
-      <c r="E29" s="68">
+      <c r="E29" s="59">
         <v>32.625</v>
       </c>
-      <c r="F29" s="67">
+      <c r="F29" s="58">
         <v>83</v>
       </c>
-      <c r="G29" s="67">
+      <c r="G29" s="58">
         <v>49.5</v>
       </c>
-      <c r="H29" s="58" t="s">
+      <c r="H29" s="49" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="30" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="79"/>
-      <c r="C30" s="77" t="s">
+      <c r="B30" s="70"/>
+      <c r="C30" s="68" t="s">
         <v>388</v>
       </c>
-      <c r="D30" s="80">
+      <c r="D30" s="71">
         <v>173.875</v>
       </c>
-      <c r="E30" s="68">
+      <c r="E30" s="59">
         <v>91.625</v>
       </c>
-      <c r="F30" s="80">
+      <c r="F30" s="71">
         <v>285.375</v>
       </c>
-      <c r="G30" s="80">
+      <c r="G30" s="71">
         <v>143</v>
       </c>
-      <c r="H30" s="58" t="s">
+      <c r="H30" s="49" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="31" spans="2:17" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="70"/>
-      <c r="C31" s="70"/>
-      <c r="D31" s="70"/>
-      <c r="E31" s="70"/>
-      <c r="F31" s="70"/>
-      <c r="G31" s="70"/>
-      <c r="H31" s="70"/>
+      <c r="B31" s="61"/>
+      <c r="C31" s="61"/>
+      <c r="D31" s="61"/>
+      <c r="E31" s="61"/>
+      <c r="F31" s="61"/>
+      <c r="G31" s="61"/>
+      <c r="H31" s="61"/>
     </row>
     <row r="32" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="81" t="s">
+      <c r="B32" s="72" t="s">
         <v>392</v>
       </c>
-      <c r="C32" s="82" t="s">
+      <c r="C32" s="73" t="s">
         <v>385</v>
       </c>
-      <c r="D32" s="83">
+      <c r="D32" s="74">
         <v>0.89655172413793105</v>
       </c>
-      <c r="E32" s="64">
+      <c r="E32" s="55">
         <v>1</v>
       </c>
-      <c r="F32" s="83">
+      <c r="F32" s="74">
         <v>0.86206896551724099</v>
       </c>
-      <c r="G32" s="83">
+      <c r="G32" s="74">
         <v>1</v>
       </c>
-      <c r="H32" s="58" t="s">
+      <c r="H32" s="49" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="33" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="84"/>
-      <c r="C33" s="66" t="s">
+      <c r="B33" s="75"/>
+      <c r="C33" s="57" t="s">
         <v>387</v>
       </c>
-      <c r="D33" s="67">
+      <c r="D33" s="58">
         <v>97.137931034482804</v>
       </c>
-      <c r="E33" s="68">
+      <c r="E33" s="59">
         <v>123.620689655172</v>
       </c>
-      <c r="F33" s="67">
+      <c r="F33" s="58">
         <v>157.241379310345</v>
       </c>
-      <c r="G33" s="67">
+      <c r="G33" s="58">
         <v>187.37931034482801</v>
       </c>
-      <c r="H33" s="57" t="s">
+      <c r="H33" s="48" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="34" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="84"/>
-      <c r="C34" s="82" t="s">
+      <c r="B34" s="75"/>
+      <c r="C34" s="73" t="s">
         <v>388</v>
       </c>
-      <c r="D34" s="85">
+      <c r="D34" s="76">
         <v>356.31034482758599</v>
       </c>
-      <c r="E34" s="68">
+      <c r="E34" s="59">
         <v>340.10344827586198</v>
       </c>
-      <c r="F34" s="85">
+      <c r="F34" s="76">
         <v>533.68965517241395</v>
       </c>
-      <c r="G34" s="85">
+      <c r="G34" s="76">
         <v>535.86206896551698</v>
       </c>
-      <c r="H34" s="58" t="s">
+      <c r="H34" s="49" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="35" spans="2:12" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="70"/>
-      <c r="C35" s="70"/>
-      <c r="D35" s="70"/>
-      <c r="E35" s="70"/>
-      <c r="F35" s="70"/>
-      <c r="G35" s="70"/>
-      <c r="H35" s="70"/>
+      <c r="B35" s="61"/>
+      <c r="C35" s="61"/>
+      <c r="D35" s="61"/>
+      <c r="E35" s="61"/>
+      <c r="F35" s="61"/>
+      <c r="G35" s="61"/>
+      <c r="H35" s="61"/>
     </row>
     <row r="37" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="26" t="s">
+      <c r="B37" s="104" t="s">
         <v>393</v>
       </c>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="26"/>
-      <c r="J37" s="26"/>
-      <c r="K37" s="26"/>
-      <c r="L37" s="26"/>
+      <c r="C37" s="104"/>
+      <c r="D37" s="104"/>
+      <c r="E37" s="104"/>
+      <c r="F37" s="104"/>
+      <c r="G37" s="104"/>
+      <c r="H37" s="104"/>
+      <c r="I37" s="104"/>
+      <c r="J37" s="104"/>
+      <c r="K37" s="104"/>
+      <c r="L37" s="104"/>
     </row>
     <row r="38" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="27" t="s">
+      <c r="B38" s="22" t="s">
         <v>381</v>
       </c>
-      <c r="C38" s="27" t="s">
+      <c r="C38" s="22" t="s">
         <v>382</v>
       </c>
-      <c r="D38" s="57" t="s">
+      <c r="D38" s="48" t="s">
         <v>386</v>
       </c>
-      <c r="E38" s="59" t="s">
+      <c r="E38" s="50" t="s">
         <v>394</v>
       </c>
-      <c r="F38" s="28" t="s">
+      <c r="F38" s="23" t="s">
         <v>395</v>
       </c>
-      <c r="G38" s="57" t="s">
+      <c r="G38" s="48" t="s">
         <v>389</v>
       </c>
-      <c r="H38" s="60" t="s">
+      <c r="H38" s="51" t="s">
         <v>396</v>
       </c>
-      <c r="I38" s="28" t="s">
+      <c r="I38" s="23" t="s">
         <v>397</v>
       </c>
     </row>
     <row r="39" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="61" t="s">
+      <c r="B39" s="52" t="s">
         <v>384</v>
       </c>
-      <c r="C39" s="62" t="s">
+      <c r="C39" s="53" t="s">
         <v>387</v>
       </c>
-      <c r="D39" s="69">
+      <c r="D39" s="60">
         <v>134.222222222222</v>
       </c>
-      <c r="E39" s="69">
+      <c r="E39" s="60">
         <v>196.666666666667</v>
       </c>
-      <c r="F39" s="64">
+      <c r="F39" s="55">
         <v>0.31751412429378501</v>
       </c>
-      <c r="G39" s="69">
+      <c r="G39" s="60">
         <v>160.777777777778</v>
       </c>
-      <c r="H39" s="69">
+      <c r="H39" s="60">
         <v>305</v>
       </c>
-      <c r="I39" s="64">
+      <c r="I39" s="55">
         <v>0.47285974499089301</v>
       </c>
     </row>
     <row r="40" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="62"/>
-      <c r="C40" s="66" t="s">
+      <c r="B40" s="53"/>
+      <c r="C40" s="57" t="s">
         <v>388</v>
       </c>
-      <c r="D40" s="67">
+      <c r="D40" s="58">
         <v>327.555555555556</v>
       </c>
-      <c r="E40" s="67">
+      <c r="E40" s="58">
         <v>509.222222222222</v>
       </c>
-      <c r="F40" s="64">
+      <c r="F40" s="55">
         <v>0.35675321841588498</v>
       </c>
-      <c r="G40" s="67">
+      <c r="G40" s="58">
         <v>324.88888888888903</v>
       </c>
-      <c r="H40" s="67">
+      <c r="H40" s="58">
         <v>640.11111111111097</v>
       </c>
-      <c r="I40" s="64">
+      <c r="I40" s="55">
         <v>0.49244922756465898</v>
       </c>
     </row>
     <row r="41" spans="2:12" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="70"/>
-      <c r="C41" s="70"/>
-      <c r="D41" s="70"/>
-      <c r="E41" s="70"/>
-      <c r="F41" s="70"/>
-      <c r="G41" s="70"/>
-      <c r="H41" s="70"/>
-      <c r="I41" s="70"/>
+      <c r="B41" s="61"/>
+      <c r="C41" s="61"/>
+      <c r="D41" s="61"/>
+      <c r="E41" s="61"/>
+      <c r="F41" s="61"/>
+      <c r="G41" s="61"/>
+      <c r="H41" s="61"/>
+      <c r="I41" s="61"/>
     </row>
     <row r="42" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="71" t="s">
+      <c r="B42" s="62" t="s">
         <v>390</v>
       </c>
-      <c r="C42" s="72" t="s">
+      <c r="C42" s="63" t="s">
         <v>387</v>
       </c>
-      <c r="D42" s="75">
+      <c r="D42" s="66">
         <v>111.333333333333</v>
       </c>
-      <c r="E42" s="75">
+      <c r="E42" s="66">
         <v>177.166666666667</v>
       </c>
-      <c r="F42" s="64">
+      <c r="F42" s="55">
         <v>0.37158984007525903</v>
       </c>
-      <c r="G42" s="75">
+      <c r="G42" s="66">
         <v>156.416666666667</v>
       </c>
-      <c r="H42" s="75">
+      <c r="H42" s="66">
         <v>191.083333333333</v>
       </c>
-      <c r="I42" s="86">
+      <c r="I42" s="77">
         <v>0.18142171827300499</v>
       </c>
     </row>
     <row r="43" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="72"/>
-      <c r="C43" s="66" t="s">
+      <c r="B43" s="63"/>
+      <c r="C43" s="57" t="s">
         <v>388</v>
       </c>
-      <c r="D43" s="67">
+      <c r="D43" s="58">
         <v>499.5</v>
       </c>
-      <c r="E43" s="67">
+      <c r="E43" s="58">
         <v>717.58333333333303</v>
       </c>
-      <c r="F43" s="64">
+      <c r="F43" s="55">
         <v>0.30391359888514702</v>
       </c>
-      <c r="G43" s="67">
+      <c r="G43" s="58">
         <v>517.16666666666697</v>
       </c>
-      <c r="H43" s="67">
+      <c r="H43" s="58">
         <v>719.58333333333303</v>
       </c>
-      <c r="I43" s="87">
+      <c r="I43" s="78">
         <v>0.28129704690214302</v>
       </c>
     </row>
     <row r="44" spans="2:12" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="70"/>
-      <c r="C44" s="70"/>
-      <c r="D44" s="70"/>
-      <c r="E44" s="70"/>
-      <c r="F44" s="70"/>
-      <c r="G44" s="70"/>
-      <c r="H44" s="70"/>
-      <c r="I44" s="70"/>
+      <c r="B44" s="61"/>
+      <c r="C44" s="61"/>
+      <c r="D44" s="61"/>
+      <c r="E44" s="61"/>
+      <c r="F44" s="61"/>
+      <c r="G44" s="61"/>
+      <c r="H44" s="61"/>
+      <c r="I44" s="61"/>
     </row>
     <row r="45" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="76" t="s">
+      <c r="B45" s="67" t="s">
         <v>391</v>
       </c>
-      <c r="C45" s="77" t="s">
+      <c r="C45" s="68" t="s">
         <v>387</v>
       </c>
-      <c r="D45" s="80">
+      <c r="D45" s="71">
         <v>34.125</v>
       </c>
-      <c r="E45" s="80">
+      <c r="E45" s="71">
         <v>83</v>
       </c>
-      <c r="F45" s="64">
+      <c r="F45" s="55">
         <v>0.58885542168674698</v>
       </c>
-      <c r="G45" s="80">
+      <c r="G45" s="71">
         <v>32.625</v>
       </c>
-      <c r="H45" s="80">
+      <c r="H45" s="71">
         <v>49.5</v>
       </c>
-      <c r="I45" s="64">
+      <c r="I45" s="55">
         <v>0.34090909090909099</v>
       </c>
     </row>
     <row r="46" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="77"/>
-      <c r="C46" s="66" t="s">
+      <c r="B46" s="68"/>
+      <c r="C46" s="57" t="s">
         <v>388</v>
       </c>
-      <c r="D46" s="67">
+      <c r="D46" s="58">
         <v>173.875</v>
       </c>
-      <c r="E46" s="67">
+      <c r="E46" s="58">
         <v>285.375</v>
       </c>
-      <c r="F46" s="64">
+      <c r="F46" s="55">
         <v>0.390713972842751</v>
       </c>
-      <c r="G46" s="67">
+      <c r="G46" s="58">
         <v>91.625</v>
       </c>
-      <c r="H46" s="67">
+      <c r="H46" s="58">
         <v>143</v>
       </c>
-      <c r="I46" s="64">
+      <c r="I46" s="55">
         <v>0.35926573426573399</v>
       </c>
     </row>
     <row r="47" spans="2:12" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="70"/>
-      <c r="C47" s="70"/>
-      <c r="D47" s="70"/>
-      <c r="E47" s="70"/>
-      <c r="F47" s="70"/>
-      <c r="G47" s="70"/>
-      <c r="H47" s="70"/>
-      <c r="I47" s="70"/>
+      <c r="B47" s="61"/>
+      <c r="C47" s="61"/>
+      <c r="D47" s="61"/>
+      <c r="E47" s="61"/>
+      <c r="F47" s="61"/>
+      <c r="G47" s="61"/>
+      <c r="H47" s="61"/>
+      <c r="I47" s="61"/>
     </row>
     <row r="48" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="81" t="s">
+      <c r="B48" s="72" t="s">
         <v>392</v>
       </c>
-      <c r="C48" s="82" t="s">
+      <c r="C48" s="73" t="s">
         <v>387</v>
       </c>
-      <c r="D48" s="85">
+      <c r="D48" s="76">
         <v>97.137931034482804</v>
       </c>
-      <c r="E48" s="85">
+      <c r="E48" s="76">
         <v>157.241379310345</v>
       </c>
-      <c r="F48" s="64">
+      <c r="F48" s="55">
         <v>0.38223684210526299</v>
       </c>
-      <c r="G48" s="85">
+      <c r="G48" s="76">
         <v>123.620689655172</v>
       </c>
-      <c r="H48" s="85">
+      <c r="H48" s="76">
         <v>187.37931034482801</v>
       </c>
-      <c r="I48" s="64">
+      <c r="I48" s="55">
         <v>0.34026499815973499</v>
       </c>
     </row>
     <row r="49" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="82"/>
-      <c r="C49" s="66" t="s">
+      <c r="B49" s="73"/>
+      <c r="C49" s="57" t="s">
         <v>388</v>
       </c>
-      <c r="D49" s="67">
+      <c r="D49" s="58">
         <v>356.31034482758599</v>
       </c>
-      <c r="E49" s="67">
+      <c r="E49" s="58">
         <v>533.68965517241395</v>
       </c>
-      <c r="F49" s="64">
+      <c r="F49" s="55">
         <v>0.332364153259676</v>
       </c>
-      <c r="G49" s="67">
+      <c r="G49" s="58">
         <v>340.10344827586198</v>
       </c>
-      <c r="H49" s="67">
+      <c r="H49" s="58">
         <v>535.86206896551698</v>
       </c>
-      <c r="I49" s="64">
+      <c r="I49" s="55">
         <v>0.36531531531531503</v>
       </c>
     </row>
     <row r="50" spans="2:11" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="70"/>
-      <c r="C50" s="70"/>
-      <c r="D50" s="70"/>
-      <c r="E50" s="70"/>
-      <c r="F50" s="70"/>
-      <c r="G50" s="70"/>
-      <c r="H50" s="70"/>
-      <c r="I50" s="70"/>
+      <c r="B50" s="61"/>
+      <c r="C50" s="61"/>
+      <c r="D50" s="61"/>
+      <c r="E50" s="61"/>
+      <c r="F50" s="61"/>
+      <c r="G50" s="61"/>
+      <c r="H50" s="61"/>
+      <c r="I50" s="61"/>
     </row>
     <row r="52" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="26" t="s">
+      <c r="B52" s="104" t="s">
         <v>398</v>
       </c>
-      <c r="C52" s="26"/>
-      <c r="D52" s="26"/>
-      <c r="E52" s="26"/>
-      <c r="F52" s="26"/>
-      <c r="G52" s="26"/>
-      <c r="H52" s="26"/>
+      <c r="C52" s="104"/>
+      <c r="D52" s="104"/>
+      <c r="E52" s="104"/>
+      <c r="F52" s="104"/>
+      <c r="G52" s="104"/>
+      <c r="H52" s="104"/>
     </row>
     <row r="53" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B53" s="27" t="s">
+      <c r="B53" s="22" t="s">
         <v>381</v>
       </c>
-      <c r="C53" s="57" t="s">
+      <c r="C53" s="48" t="s">
         <v>359</v>
       </c>
-      <c r="D53" s="58" t="s">
+      <c r="D53" s="49" t="s">
         <v>361</v>
       </c>
-      <c r="E53" s="59" t="s">
+      <c r="E53" s="50" t="s">
         <v>366</v>
       </c>
-      <c r="F53" s="60" t="s">
+      <c r="F53" s="51" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="54" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B54" s="88" t="s">
+      <c r="B54" s="79" t="s">
         <v>384</v>
       </c>
-      <c r="C54" s="89">
+      <c r="C54" s="80">
         <v>1</v>
       </c>
-      <c r="D54" s="90">
+      <c r="D54" s="81">
         <v>1</v>
       </c>
-      <c r="E54" s="89">
+      <c r="E54" s="80">
         <v>0.88888888888888895</v>
       </c>
-      <c r="F54" s="89">
+      <c r="F54" s="80">
         <v>1</v>
       </c>
     </row>
     <row r="55" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="66" t="s">
+      <c r="B55" s="57" t="s">
         <v>390</v>
       </c>
-      <c r="C55" s="91">
+      <c r="C55" s="82">
         <v>0.83333333333333304</v>
       </c>
-      <c r="D55" s="90">
+      <c r="D55" s="81">
         <v>1</v>
       </c>
-      <c r="E55" s="91">
+      <c r="E55" s="82">
         <v>0.83333333333333304</v>
       </c>
-      <c r="F55" s="91">
+      <c r="F55" s="82">
         <v>1</v>
       </c>
     </row>
     <row r="56" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="88" t="s">
+      <c r="B56" s="79" t="s">
         <v>391</v>
       </c>
-      <c r="C56" s="89">
+      <c r="C56" s="80">
         <v>0.875</v>
       </c>
-      <c r="D56" s="90">
+      <c r="D56" s="81">
         <v>1</v>
       </c>
-      <c r="E56" s="89">
+      <c r="E56" s="80">
         <v>0.875</v>
       </c>
-      <c r="F56" s="89">
+      <c r="F56" s="80">
         <v>1</v>
       </c>
     </row>
     <row r="57" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B57" s="66" t="s">
+      <c r="B57" s="57" t="s">
         <v>399</v>
       </c>
-      <c r="C57" s="91">
+      <c r="C57" s="82">
         <v>0.89655172413793105</v>
       </c>
-      <c r="D57" s="90">
+      <c r="D57" s="81">
         <v>1</v>
       </c>
-      <c r="E57" s="91">
+      <c r="E57" s="82">
         <v>0.86206896551724099</v>
       </c>
-      <c r="F57" s="91">
+      <c r="F57" s="82">
         <v>1</v>
       </c>
     </row>
     <row r="60" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="26" t="s">
+      <c r="B60" s="104" t="s">
         <v>400</v>
       </c>
-      <c r="C60" s="26"/>
-      <c r="D60" s="26"/>
-      <c r="E60" s="26"/>
-      <c r="F60" s="26"/>
-      <c r="G60" s="26"/>
-      <c r="H60" s="26"/>
+      <c r="C60" s="104"/>
+      <c r="D60" s="104"/>
+      <c r="E60" s="104"/>
+      <c r="F60" s="104"/>
+      <c r="G60" s="104"/>
+      <c r="H60" s="104"/>
     </row>
     <row r="61" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="27" t="s">
+      <c r="B61" s="22" t="s">
         <v>381</v>
       </c>
-      <c r="C61" s="57" t="s">
+      <c r="C61" s="48" t="s">
         <v>359</v>
       </c>
-      <c r="D61" s="58" t="s">
+      <c r="D61" s="49" t="s">
         <v>361</v>
       </c>
-      <c r="E61" s="59" t="s">
+      <c r="E61" s="50" t="s">
         <v>366</v>
       </c>
-      <c r="F61" s="60" t="s">
+      <c r="F61" s="51" t="s">
         <v>368</v>
       </c>
-      <c r="G61" s="27" t="s">
+      <c r="G61" s="22" t="s">
         <v>381</v>
       </c>
-      <c r="H61" s="57" t="s">
+      <c r="H61" s="48" t="s">
         <v>359</v>
       </c>
-      <c r="I61" s="58" t="s">
+      <c r="I61" s="49" t="s">
         <v>361</v>
       </c>
-      <c r="J61" s="59" t="s">
+      <c r="J61" s="50" t="s">
         <v>366</v>
       </c>
-      <c r="K61" s="60" t="s">
+      <c r="K61" s="51" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="62" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="88" t="s">
+      <c r="B62" s="79" t="s">
         <v>384</v>
       </c>
-      <c r="C62" s="92">
+      <c r="C62" s="83">
         <v>134.222222222222</v>
       </c>
-      <c r="D62" s="68">
+      <c r="D62" s="59">
         <v>160.777777777778</v>
       </c>
-      <c r="E62" s="92">
+      <c r="E62" s="83">
         <v>196.666666666667</v>
       </c>
-      <c r="F62" s="92">
+      <c r="F62" s="83">
         <v>305</v>
       </c>
-      <c r="G62" s="88" t="s">
+      <c r="G62" s="79" t="s">
         <v>384</v>
       </c>
-      <c r="H62" s="92">
+      <c r="H62" s="83">
         <v>327.555555555556</v>
       </c>
-      <c r="I62" s="68">
+      <c r="I62" s="59">
         <v>324.88888888888903</v>
       </c>
-      <c r="J62" s="92">
+      <c r="J62" s="83">
         <v>509.222222222222</v>
       </c>
-      <c r="K62" s="92">
+      <c r="K62" s="83">
         <v>640.11111111111097</v>
       </c>
     </row>
     <row r="63" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="66" t="s">
+      <c r="B63" s="57" t="s">
         <v>390</v>
       </c>
-      <c r="C63" s="67">
+      <c r="C63" s="58">
         <v>111.333333333333</v>
       </c>
-      <c r="D63" s="68">
+      <c r="D63" s="59">
         <v>156.416666666667</v>
       </c>
-      <c r="E63" s="67">
+      <c r="E63" s="58">
         <v>177.166666666667</v>
       </c>
-      <c r="F63" s="67">
+      <c r="F63" s="58">
         <v>191.083333333333</v>
       </c>
-      <c r="G63" s="66" t="s">
+      <c r="G63" s="57" t="s">
         <v>390</v>
       </c>
-      <c r="H63" s="67">
+      <c r="H63" s="58">
         <v>499.5</v>
       </c>
-      <c r="I63" s="68">
+      <c r="I63" s="59">
         <v>517.16666666666697</v>
       </c>
-      <c r="J63" s="67">
+      <c r="J63" s="58">
         <v>717.58333333333303</v>
       </c>
-      <c r="K63" s="67">
+      <c r="K63" s="58">
         <v>719.58333333333303</v>
       </c>
     </row>
     <row r="64" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="88" t="s">
+      <c r="B64" s="79" t="s">
         <v>391</v>
       </c>
-      <c r="C64" s="92">
+      <c r="C64" s="83">
         <v>34.125</v>
       </c>
-      <c r="D64" s="68">
+      <c r="D64" s="59">
         <v>32.625</v>
       </c>
-      <c r="E64" s="92">
+      <c r="E64" s="83">
         <v>83</v>
       </c>
-      <c r="F64" s="92">
+      <c r="F64" s="83">
         <v>49.5</v>
       </c>
-      <c r="G64" s="88" t="s">
+      <c r="G64" s="79" t="s">
         <v>391</v>
       </c>
-      <c r="H64" s="92">
+      <c r="H64" s="83">
         <v>173.875</v>
       </c>
-      <c r="I64" s="68">
+      <c r="I64" s="59">
         <v>91.625</v>
       </c>
-      <c r="J64" s="92">
+      <c r="J64" s="83">
         <v>285.375</v>
       </c>
-      <c r="K64" s="92">
+      <c r="K64" s="83">
         <v>143</v>
       </c>
     </row>
     <row r="65" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="66" t="s">
+      <c r="B65" s="57" t="s">
         <v>399</v>
       </c>
-      <c r="C65" s="67">
+      <c r="C65" s="58">
         <v>97.137931034482804</v>
       </c>
-      <c r="D65" s="68">
+      <c r="D65" s="59">
         <v>123.620689655172</v>
       </c>
-      <c r="E65" s="67">
+      <c r="E65" s="58">
         <v>157.241379310345</v>
       </c>
-      <c r="F65" s="67">
+      <c r="F65" s="58">
         <v>187.37931034482801</v>
       </c>
-      <c r="G65" s="66" t="s">
+      <c r="G65" s="57" t="s">
         <v>399</v>
       </c>
-      <c r="H65" s="67">
+      <c r="H65" s="58">
         <v>356.31034482758599</v>
       </c>
-      <c r="I65" s="68">
+      <c r="I65" s="59">
         <v>340.10344827586198</v>
       </c>
-      <c r="J65" s="67">
+      <c r="J65" s="58">
         <v>533.68965517241395</v>
       </c>
-      <c r="K65" s="67">
+      <c r="K65" s="58">
         <v>535.86206896551698</v>
       </c>
     </row>
     <row r="68" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="26" t="s">
+      <c r="B68" s="104" t="s">
         <v>401</v>
       </c>
-      <c r="C68" s="26"/>
-      <c r="D68" s="26"/>
-      <c r="E68" s="26"/>
-      <c r="F68" s="26"/>
-      <c r="G68" s="26"/>
-      <c r="H68" s="26"/>
+      <c r="C68" s="104"/>
+      <c r="D68" s="104"/>
+      <c r="E68" s="104"/>
+      <c r="F68" s="104"/>
+      <c r="G68" s="104"/>
+      <c r="H68" s="104"/>
     </row>
     <row r="69" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="27" t="s">
+      <c r="B69" s="22" t="s">
         <v>402</v>
       </c>
-      <c r="C69" s="27" t="s">
+      <c r="C69" s="22" t="s">
         <v>381</v>
       </c>
-      <c r="D69" s="57" t="s">
+      <c r="D69" s="48" t="s">
         <v>359</v>
       </c>
-      <c r="E69" s="58" t="s">
+      <c r="E69" s="49" t="s">
         <v>361</v>
       </c>
-      <c r="F69" s="59" t="s">
+      <c r="F69" s="50" t="s">
         <v>366</v>
       </c>
-      <c r="G69" s="60" t="s">
+      <c r="G69" s="51" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="70" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="93" t="s">
+      <c r="B70" s="84" t="s">
         <v>325</v>
       </c>
-      <c r="C70" s="94" t="s">
+      <c r="C70" s="85" t="s">
         <v>403</v>
       </c>
-      <c r="D70" s="95" t="s">
+      <c r="D70" s="86" t="s">
         <v>404</v>
       </c>
-      <c r="E70" s="95" t="s">
+      <c r="E70" s="86" t="s">
         <v>404</v>
       </c>
-      <c r="F70" s="96">
+      <c r="F70" s="87">
         <v>1.3450000000000001E-3</v>
       </c>
-      <c r="G70" s="95" t="s">
+      <c r="G70" s="86" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="71" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="97" t="s">
+      <c r="B71" s="88" t="s">
         <v>405</v>
       </c>
-      <c r="C71" s="98" t="s">
+      <c r="C71" s="89" t="s">
         <v>403</v>
       </c>
-      <c r="D71" s="96">
+      <c r="D71" s="87">
         <v>5.3E-3</v>
       </c>
-      <c r="E71" s="95" t="s">
+      <c r="E71" s="86" t="s">
         <v>404</v>
       </c>
-      <c r="F71" s="95" t="s">
+      <c r="F71" s="86" t="s">
         <v>404</v>
       </c>
-      <c r="G71" s="95" t="s">
+      <c r="G71" s="86" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="72" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B72" s="93" t="s">
+      <c r="B72" s="84" t="s">
         <v>406</v>
       </c>
-      <c r="C72" s="94" t="s">
+      <c r="C72" s="85" t="s">
         <v>403</v>
       </c>
-      <c r="D72" s="96">
+      <c r="D72" s="87">
         <v>1.284E-3</v>
       </c>
-      <c r="E72" s="95" t="s">
+      <c r="E72" s="86" t="s">
         <v>404</v>
       </c>
-      <c r="F72" s="96">
+      <c r="F72" s="87">
         <v>1.284E-3</v>
       </c>
-      <c r="G72" s="95" t="s">
+      <c r="G72" s="86" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="73" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="97" t="s">
+      <c r="B73" s="88" t="s">
         <v>407</v>
       </c>
-      <c r="C73" s="98" t="s">
+      <c r="C73" s="89" t="s">
         <v>408</v>
       </c>
-      <c r="D73" s="96">
+      <c r="D73" s="87">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="E73" s="95" t="s">
+      <c r="E73" s="86" t="s">
         <v>404</v>
       </c>
-      <c r="F73" s="95" t="s">
+      <c r="F73" s="86" t="s">
         <v>404</v>
       </c>
-      <c r="G73" s="95" t="s">
+      <c r="G73" s="86" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="74" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B74" s="93" t="s">
+      <c r="B74" s="84" t="s">
         <v>409</v>
       </c>
-      <c r="C74" s="94" t="s">
+      <c r="C74" s="85" t="s">
         <v>408</v>
       </c>
-      <c r="D74" s="95" t="s">
+      <c r="D74" s="86" t="s">
         <v>404</v>
       </c>
-      <c r="E74" s="95" t="s">
+      <c r="E74" s="86" t="s">
         <v>404</v>
       </c>
-      <c r="F74" s="96">
+      <c r="F74" s="87">
         <v>0.1</v>
       </c>
-      <c r="G74" s="95" t="s">
+      <c r="G74" s="86" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="77" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="52" t="s">
+      <c r="B77" s="105" t="s">
         <v>410</v>
       </c>
-      <c r="C77" s="52"/>
-      <c r="D77" s="52"/>
-      <c r="E77" s="52"/>
-      <c r="F77" s="52"/>
+      <c r="C77" s="105"/>
+      <c r="D77" s="105"/>
+      <c r="E77" s="105"/>
+      <c r="F77" s="105"/>
     </row>
     <row r="78" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B78" s="57" t="s">
+      <c r="B78" s="48" t="s">
         <v>386</v>
       </c>
-      <c r="C78" s="99" t="s">
+      <c r="C78" s="103" t="s">
         <v>359</v>
       </c>
-      <c r="D78" s="99"/>
-      <c r="E78" s="99"/>
-      <c r="F78" s="99"/>
+      <c r="D78" s="103"/>
+      <c r="E78" s="103"/>
+      <c r="F78" s="103"/>
     </row>
     <row r="79" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B79" s="58" t="s">
+      <c r="B79" s="49" t="s">
         <v>389</v>
       </c>
-      <c r="C79" s="99" t="s">
+      <c r="C79" s="103" t="s">
         <v>361</v>
       </c>
-      <c r="D79" s="99"/>
-      <c r="E79" s="99"/>
-      <c r="F79" s="99"/>
+      <c r="D79" s="103"/>
+      <c r="E79" s="103"/>
+      <c r="F79" s="103"/>
     </row>
     <row r="80" spans="2:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B80" s="59" t="s">
+      <c r="B80" s="50" t="s">
         <v>394</v>
       </c>
-      <c r="C80" s="99" t="s">
+      <c r="C80" s="103" t="s">
         <v>366</v>
       </c>
-      <c r="D80" s="99"/>
-      <c r="E80" s="99"/>
-      <c r="F80" s="99"/>
+      <c r="D80" s="103"/>
+      <c r="E80" s="103"/>
+      <c r="F80" s="103"/>
     </row>
     <row r="81" spans="2:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B81" s="60" t="s">
+      <c r="B81" s="51" t="s">
         <v>396</v>
       </c>
-      <c r="C81" s="99" t="s">
+      <c r="C81" s="103" t="s">
         <v>368</v>
       </c>
-      <c r="D81" s="99"/>
-      <c r="E81" s="99"/>
-      <c r="F81" s="99"/>
+      <c r="D81" s="103"/>
+      <c r="E81" s="103"/>
+      <c r="F81" s="103"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="B52:H52"/>
+    <mergeCell ref="B1:R1"/>
+    <mergeCell ref="B2:R2"/>
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="C12:L12"/>
+    <mergeCell ref="C13:L13"/>
+    <mergeCell ref="C14:L14"/>
+    <mergeCell ref="C15:L15"/>
+    <mergeCell ref="C16:L16"/>
+    <mergeCell ref="B18:Q18"/>
+    <mergeCell ref="B37:L37"/>
     <mergeCell ref="C81:F81"/>
     <mergeCell ref="B60:H60"/>
     <mergeCell ref="B68:H68"/>
@@ -18752,18 +18886,6 @@
     <mergeCell ref="C78:F78"/>
     <mergeCell ref="C79:F79"/>
     <mergeCell ref="C80:F80"/>
-    <mergeCell ref="C14:L14"/>
-    <mergeCell ref="C15:L15"/>
-    <mergeCell ref="C16:L16"/>
-    <mergeCell ref="B18:Q18"/>
-    <mergeCell ref="B37:L37"/>
-    <mergeCell ref="B52:H52"/>
-    <mergeCell ref="B1:R1"/>
-    <mergeCell ref="B2:R2"/>
-    <mergeCell ref="B4:L4"/>
-    <mergeCell ref="B11:L11"/>
-    <mergeCell ref="C12:L12"/>
-    <mergeCell ref="C13:L13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -18772,248 +18894,1776 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7729A820-E01A-4B4F-BEC5-72896FA52F21}">
-  <dimension ref="A1:B30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6381B92-E053-4233-81A5-0B655C210782}">
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>446</v>
+      </c>
+      <c r="B1" t="s">
+        <v>447</v>
+      </c>
+      <c r="C1" t="s">
+        <v>448</v>
+      </c>
+      <c r="D1" t="s">
+        <v>449</v>
+      </c>
+      <c r="E1" t="s">
+        <v>447</v>
+      </c>
+      <c r="F1">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s">
+        <v>450</v>
+      </c>
+      <c r="H1" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D2" t="s">
+        <v>452</v>
+      </c>
+      <c r="E2" t="s">
+        <v>447</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s">
+        <v>450</v>
+      </c>
+      <c r="H2" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>241</v>
+      </c>
+      <c r="B3" t="s">
+        <v>447</v>
+      </c>
+      <c r="C3" t="s">
+        <v>448</v>
+      </c>
+      <c r="D3" t="s">
+        <v>453</v>
+      </c>
+      <c r="E3" t="s">
+        <v>447</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
+        <v>450</v>
+      </c>
+      <c r="H3" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B4" t="s">
+        <v>447</v>
+      </c>
+      <c r="C4" t="s">
+        <v>448</v>
+      </c>
+      <c r="D4" t="s">
+        <v>454</v>
+      </c>
+      <c r="E4" t="s">
+        <v>447</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
+        <v>450</v>
+      </c>
+      <c r="H4" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>255</v>
+      </c>
+      <c r="B5" t="s">
+        <v>447</v>
+      </c>
+      <c r="C5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D5" t="s">
+        <v>455</v>
+      </c>
+      <c r="E5" t="s">
+        <v>447</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5" t="s">
+        <v>450</v>
+      </c>
+      <c r="H5" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>262</v>
+      </c>
+      <c r="B6" t="s">
+        <v>447</v>
+      </c>
+      <c r="C6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D6" t="s">
+        <v>456</v>
+      </c>
+      <c r="E6" t="s">
+        <v>447</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>450</v>
+      </c>
+      <c r="H6" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>269</v>
+      </c>
+      <c r="B7" t="s">
+        <v>447</v>
+      </c>
+      <c r="C7" t="s">
+        <v>448</v>
+      </c>
+      <c r="D7" t="s">
+        <v>457</v>
+      </c>
+      <c r="E7" t="s">
+        <v>447</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
+        <v>450</v>
+      </c>
+      <c r="H7" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>276</v>
+      </c>
+      <c r="B8" t="s">
+        <v>447</v>
+      </c>
+      <c r="C8" t="s">
+        <v>448</v>
+      </c>
+      <c r="D8" t="s">
+        <v>458</v>
+      </c>
+      <c r="E8" t="s">
+        <v>447</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8" t="s">
+        <v>450</v>
+      </c>
+      <c r="H8" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>283</v>
+      </c>
+      <c r="B9" t="s">
+        <v>447</v>
+      </c>
+      <c r="C9" t="s">
+        <v>448</v>
+      </c>
+      <c r="D9" t="s">
+        <v>459</v>
+      </c>
+      <c r="E9" t="s">
+        <v>447</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9" t="s">
+        <v>450</v>
+      </c>
+      <c r="H9" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>290</v>
+      </c>
+      <c r="B10" t="s">
+        <v>447</v>
+      </c>
+      <c r="C10" t="s">
+        <v>448</v>
+      </c>
+      <c r="D10" t="s">
+        <v>460</v>
+      </c>
+      <c r="E10" t="s">
+        <v>447</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10" t="s">
+        <v>450</v>
+      </c>
+      <c r="H10" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>297</v>
+      </c>
+      <c r="B11" t="s">
+        <v>447</v>
+      </c>
+      <c r="C11" t="s">
+        <v>448</v>
+      </c>
+      <c r="D11" t="s">
+        <v>461</v>
+      </c>
+      <c r="E11" t="s">
+        <v>447</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11" t="s">
+        <v>450</v>
+      </c>
+      <c r="H11" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>304</v>
+      </c>
+      <c r="B12" t="s">
+        <v>447</v>
+      </c>
+      <c r="C12" t="s">
+        <v>448</v>
+      </c>
+      <c r="D12" t="s">
+        <v>462</v>
+      </c>
+      <c r="E12" t="s">
+        <v>447</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12" t="s">
+        <v>450</v>
+      </c>
+      <c r="H12" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>311</v>
+      </c>
+      <c r="B13" t="s">
+        <v>447</v>
+      </c>
+      <c r="C13" t="s">
+        <v>448</v>
+      </c>
+      <c r="D13" t="s">
+        <v>463</v>
+      </c>
+      <c r="E13" t="s">
+        <v>447</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13" t="s">
+        <v>450</v>
+      </c>
+      <c r="H13" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>318</v>
+      </c>
+      <c r="B14" t="s">
+        <v>447</v>
+      </c>
+      <c r="C14" t="s">
+        <v>448</v>
+      </c>
+      <c r="D14" t="s">
+        <v>464</v>
+      </c>
+      <c r="E14" t="s">
+        <v>447</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14" t="s">
+        <v>450</v>
+      </c>
+      <c r="H14" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>325</v>
+      </c>
+      <c r="B15" t="s">
+        <v>447</v>
+      </c>
+      <c r="C15" t="s">
+        <v>448</v>
+      </c>
+      <c r="D15" t="s">
+        <v>465</v>
+      </c>
+      <c r="E15" t="s">
+        <v>447</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15" t="s">
+        <v>450</v>
+      </c>
+      <c r="H15" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>466</v>
+      </c>
+      <c r="B16" t="s">
+        <v>447</v>
+      </c>
+      <c r="C16" t="s">
+        <v>448</v>
+      </c>
+      <c r="D16" t="s">
+        <v>467</v>
+      </c>
+      <c r="E16" t="s">
+        <v>447</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16" t="s">
+        <v>450</v>
+      </c>
+      <c r="H16" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>468</v>
+      </c>
+      <c r="B17" t="s">
+        <v>447</v>
+      </c>
+      <c r="C17" t="s">
+        <v>448</v>
+      </c>
+      <c r="D17" t="s">
+        <v>469</v>
+      </c>
+      <c r="E17" t="s">
+        <v>447</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17" t="s">
+        <v>450</v>
+      </c>
+      <c r="H17" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>470</v>
+      </c>
+      <c r="B18" t="s">
+        <v>447</v>
+      </c>
+      <c r="C18" t="s">
+        <v>448</v>
+      </c>
+      <c r="D18" t="s">
+        <v>471</v>
+      </c>
+      <c r="E18" t="s">
+        <v>447</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18" t="s">
+        <v>450</v>
+      </c>
+      <c r="H18" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>405</v>
+      </c>
+      <c r="B19" t="s">
+        <v>447</v>
+      </c>
+      <c r="C19" t="s">
+        <v>448</v>
+      </c>
+      <c r="D19" t="s">
+        <v>472</v>
+      </c>
+      <c r="E19" t="s">
+        <v>447</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19" t="s">
+        <v>450</v>
+      </c>
+      <c r="H19" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>406</v>
+      </c>
+      <c r="B20" t="s">
+        <v>447</v>
+      </c>
+      <c r="C20" t="s">
+        <v>448</v>
+      </c>
+      <c r="D20" t="s">
+        <v>473</v>
+      </c>
+      <c r="E20" t="s">
+        <v>447</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20" t="s">
+        <v>450</v>
+      </c>
+      <c r="H20" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>474</v>
+      </c>
+      <c r="B21" t="s">
+        <v>447</v>
+      </c>
+      <c r="C21" t="s">
+        <v>448</v>
+      </c>
+      <c r="D21" t="s">
+        <v>475</v>
+      </c>
+      <c r="E21" t="s">
+        <v>447</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21" t="s">
+        <v>450</v>
+      </c>
+      <c r="H21" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>407</v>
+      </c>
+      <c r="B22" t="s">
+        <v>447</v>
+      </c>
+      <c r="C22" t="s">
+        <v>448</v>
+      </c>
+      <c r="D22" t="s">
+        <v>476</v>
+      </c>
+      <c r="E22" t="s">
+        <v>447</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22" t="s">
+        <v>450</v>
+      </c>
+      <c r="H22" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>409</v>
+      </c>
+      <c r="B23" t="s">
+        <v>447</v>
+      </c>
+      <c r="C23" t="s">
+        <v>448</v>
+      </c>
+      <c r="D23" t="s">
+        <v>477</v>
+      </c>
+      <c r="E23" t="s">
+        <v>447</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23" t="s">
+        <v>450</v>
+      </c>
+      <c r="H23" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>478</v>
+      </c>
+      <c r="B24" t="s">
+        <v>447</v>
+      </c>
+      <c r="C24" t="s">
+        <v>448</v>
+      </c>
+      <c r="D24" t="s">
+        <v>479</v>
+      </c>
+      <c r="E24" t="s">
+        <v>447</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24" t="s">
+        <v>450</v>
+      </c>
+      <c r="H24" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>480</v>
+      </c>
+      <c r="B25" t="s">
+        <v>447</v>
+      </c>
+      <c r="C25" t="s">
+        <v>448</v>
+      </c>
+      <c r="D25" t="s">
+        <v>481</v>
+      </c>
+      <c r="E25" t="s">
+        <v>447</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25" t="s">
+        <v>450</v>
+      </c>
+      <c r="H25" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>482</v>
+      </c>
+      <c r="B26" t="s">
+        <v>447</v>
+      </c>
+      <c r="C26" t="s">
+        <v>448</v>
+      </c>
+      <c r="D26" t="s">
+        <v>483</v>
+      </c>
+      <c r="E26" t="s">
+        <v>447</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26" t="s">
+        <v>450</v>
+      </c>
+      <c r="H26" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>484</v>
+      </c>
+      <c r="B27" t="s">
+        <v>447</v>
+      </c>
+      <c r="C27" t="s">
+        <v>448</v>
+      </c>
+      <c r="D27" t="s">
+        <v>485</v>
+      </c>
+      <c r="E27" t="s">
+        <v>447</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" t="s">
+        <v>450</v>
+      </c>
+      <c r="H27" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>486</v>
+      </c>
+      <c r="B28" t="s">
+        <v>447</v>
+      </c>
+      <c r="C28" t="s">
+        <v>448</v>
+      </c>
+      <c r="D28" t="s">
+        <v>487</v>
+      </c>
+      <c r="E28" t="s">
+        <v>447</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28" t="s">
+        <v>450</v>
+      </c>
+      <c r="H28" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>488</v>
+      </c>
+      <c r="B29" t="s">
+        <v>447</v>
+      </c>
+      <c r="C29" t="s">
+        <v>448</v>
+      </c>
+      <c r="D29" t="s">
+        <v>489</v>
+      </c>
+      <c r="E29" t="s">
+        <v>447</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29" t="s">
+        <v>450</v>
+      </c>
+      <c r="H29" t="s">
+        <v>451</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{085F676F-525D-4676-9613-88ED455FD340}">
+  <dimension ref="A2:D31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>508</v>
+      </c>
+      <c r="B2" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>446</v>
+      </c>
+      <c r="B3" s="93">
+        <v>362.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B4" s="93">
+        <v>362.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>241</v>
+      </c>
+      <c r="B5" s="93">
+        <v>361.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>248</v>
+      </c>
+      <c r="B6" s="93">
+        <v>362.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>255</v>
+      </c>
+      <c r="B7" s="93">
+        <v>362.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>262</v>
+      </c>
+      <c r="B8" s="93">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>269</v>
+      </c>
+      <c r="B9" s="93">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>276</v>
+      </c>
+      <c r="B10" s="93">
+        <v>772.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>283</v>
+      </c>
+      <c r="B11" s="93">
+        <v>629.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>290</v>
+      </c>
+      <c r="B12" s="96">
+        <v>903.7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>297</v>
+      </c>
+      <c r="B13" s="96">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>304</v>
+      </c>
+      <c r="B14" s="96">
+        <v>711.1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>311</v>
+      </c>
+      <c r="B15" s="96">
+        <v>622.20000000000005</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>318</v>
+      </c>
+      <c r="B16" s="96">
+        <v>790.4</v>
+      </c>
+      <c r="D16" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>325</v>
+      </c>
+      <c r="B17" s="96">
+        <v>697</v>
+      </c>
+      <c r="D17" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>466</v>
+      </c>
+      <c r="B18" s="96">
+        <v>714.4</v>
+      </c>
+      <c r="D18" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>468</v>
+      </c>
+      <c r="B19" s="96">
+        <v>636.9</v>
+      </c>
+      <c r="D19" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>470</v>
+      </c>
+      <c r="B20" s="96">
+        <v>990.1</v>
+      </c>
+      <c r="D20" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>405</v>
+      </c>
+      <c r="B21" s="96">
+        <v>840.1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>406</v>
+      </c>
+      <c r="B22" s="96">
+        <v>737</v>
+      </c>
+      <c r="D22" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>474</v>
+      </c>
+      <c r="B23" s="96">
+        <v>545.79999999999995</v>
+      </c>
+      <c r="D23" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>407</v>
+      </c>
+      <c r="B24" s="99">
+        <v>885.6</v>
+      </c>
+      <c r="D24" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>409</v>
+      </c>
+      <c r="B25" s="99">
+        <v>741.4</v>
+      </c>
+      <c r="D25" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>478</v>
+      </c>
+      <c r="B26" s="99">
+        <v>642.70000000000005</v>
+      </c>
+      <c r="D26" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>480</v>
+      </c>
+      <c r="B27" s="99">
+        <v>598.1</v>
+      </c>
+      <c r="D27" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>482</v>
+      </c>
+      <c r="B28" s="99">
+        <v>1223.2</v>
+      </c>
+      <c r="D28" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>484</v>
+      </c>
+      <c r="B29" s="99">
+        <v>1083.0999999999999</v>
+      </c>
+      <c r="D29" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>486</v>
+      </c>
+      <c r="B30" s="99">
+        <v>1083.0999999999999</v>
+      </c>
+      <c r="D30" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>488</v>
+      </c>
+      <c r="B31" s="99">
+        <v>1081.0999999999999</v>
+      </c>
+      <c r="D31" t="s">
+        <v>507</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7729A820-E01A-4B4F-BEC5-72896FA52F21}">
+  <dimension ref="A1:J31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>490</v>
+      </c>
+      <c r="B1">
+        <v>25</v>
+      </c>
+      <c r="D1" s="100" t="s">
+        <v>490</v>
+      </c>
+      <c r="E1" s="100">
+        <v>50</v>
+      </c>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="D2" s="100" t="s">
+        <v>412</v>
+      </c>
+      <c r="E2" s="100" t="s">
+        <v>413</v>
+      </c>
+      <c r="F2" s="100" t="s">
+        <v>414</v>
+      </c>
+      <c r="G2" s="100" t="s">
+        <v>415</v>
+      </c>
+      <c r="J2" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>218</v>
       </c>
-      <c r="B2" s="15">
+      <c r="B3" s="15">
         <v>191.3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="D3" s="91" t="s">
+        <v>416</v>
+      </c>
+      <c r="E3" s="92" t="s">
+        <v>417</v>
+      </c>
+      <c r="F3" s="93">
+        <v>362.4</v>
+      </c>
+      <c r="G3" s="93">
+        <v>362.4</v>
+      </c>
+      <c r="J3" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>234</v>
-      </c>
-      <c r="B3" s="15">
-        <v>190.3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>241</v>
       </c>
       <c r="B4" s="15">
         <v>190.3</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D4" s="91" t="s">
+        <v>418</v>
+      </c>
+      <c r="E4" s="92" t="s">
+        <v>417</v>
+      </c>
+      <c r="F4" s="93">
+        <v>362.4</v>
+      </c>
+      <c r="G4" s="93">
+        <v>362.4</v>
+      </c>
+      <c r="J4" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>241</v>
+      </c>
+      <c r="B5" s="15">
+        <v>190.3</v>
+      </c>
+      <c r="D5" s="91" t="s">
+        <v>419</v>
+      </c>
+      <c r="E5" s="92" t="s">
+        <v>417</v>
+      </c>
+      <c r="F5" s="93">
+        <v>361.4</v>
+      </c>
+      <c r="G5" s="93">
+        <v>361.4</v>
+      </c>
+      <c r="J5" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>248</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B6" s="15">
         <v>186.9</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="D6" s="91" t="s">
+        <v>420</v>
+      </c>
+      <c r="E6" s="92" t="s">
+        <v>417</v>
+      </c>
+      <c r="F6" s="93">
+        <v>362.4</v>
+      </c>
+      <c r="G6" s="93">
+        <v>362.4</v>
+      </c>
+      <c r="J6" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>255</v>
-      </c>
-      <c r="B6" s="15">
-        <v>191.3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>262</v>
       </c>
       <c r="B7" s="15">
         <v>191.3</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D7" s="91" t="s">
+        <v>421</v>
+      </c>
+      <c r="E7" s="92" t="s">
+        <v>417</v>
+      </c>
+      <c r="F7" s="93">
+        <v>362.4</v>
+      </c>
+      <c r="G7" s="93">
+        <v>362.4</v>
+      </c>
+      <c r="J7" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="B8" s="15">
         <v>191.3</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D8" s="91" t="s">
+        <v>422</v>
+      </c>
+      <c r="E8" s="92" t="s">
+        <v>417</v>
+      </c>
+      <c r="F8" s="93">
+        <v>1044</v>
+      </c>
+      <c r="G8" s="93">
+        <v>1043.3</v>
+      </c>
+      <c r="J8" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>269</v>
+      </c>
+      <c r="B9" s="15">
+        <v>191.3</v>
+      </c>
+      <c r="D9" s="91" t="s">
+        <v>423</v>
+      </c>
+      <c r="E9" s="92" t="s">
+        <v>417</v>
+      </c>
+      <c r="F9" s="93">
+        <v>909</v>
+      </c>
+      <c r="G9" s="93">
+        <v>909</v>
+      </c>
+      <c r="J9" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>276</v>
-      </c>
-      <c r="B9" s="18">
-        <v>191.3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>283</v>
       </c>
       <c r="B10" s="18">
         <v>191.3</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D10" s="91" t="s">
+        <v>424</v>
+      </c>
+      <c r="E10" s="92" t="s">
+        <v>417</v>
+      </c>
+      <c r="F10" s="93">
+        <v>772.9</v>
+      </c>
+      <c r="G10" s="93">
+        <v>769.2</v>
+      </c>
+      <c r="J10" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>283</v>
+      </c>
+      <c r="B11" s="18">
+        <v>191.3</v>
+      </c>
+      <c r="D11" s="91" t="s">
+        <v>425</v>
+      </c>
+      <c r="E11" s="92" t="s">
+        <v>417</v>
+      </c>
+      <c r="F11" s="93">
+        <v>629.4</v>
+      </c>
+      <c r="G11" s="93">
+        <v>619.1</v>
+      </c>
+      <c r="J11" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>290</v>
       </c>
-      <c r="B11" s="19">
+      <c r="B12" s="19">
         <v>617.1</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="D12" s="94" t="s">
+        <v>426</v>
+      </c>
+      <c r="E12" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F12" s="96">
+        <v>903.7</v>
+      </c>
+      <c r="G12" s="96">
+        <v>892.1</v>
+      </c>
+      <c r="J12" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>297</v>
       </c>
-      <c r="B12" s="18">
+      <c r="B13" s="18">
         <v>547.1</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="D13" s="94" t="s">
+        <v>427</v>
+      </c>
+      <c r="E13" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F13" s="96">
+        <v>793</v>
+      </c>
+      <c r="G13" s="96">
+        <v>791.3</v>
+      </c>
+      <c r="J13" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>304</v>
       </c>
-      <c r="B13" s="18">
+      <c r="B14" s="18">
         <v>454.6</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="D14" s="94" t="s">
+        <v>428</v>
+      </c>
+      <c r="E14" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F14" s="96">
+        <v>711.1</v>
+      </c>
+      <c r="G14" s="96">
+        <v>707.2</v>
+      </c>
+      <c r="J14" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>311</v>
       </c>
-      <c r="B14" s="18">
+      <c r="B15" s="18">
         <v>416.9</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="D15" s="94" t="s">
+        <v>429</v>
+      </c>
+      <c r="E15" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F15" s="96">
+        <v>622.20000000000005</v>
+      </c>
+      <c r="G15" s="96">
+        <v>594.70000000000005</v>
+      </c>
+      <c r="J15" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>318</v>
       </c>
-      <c r="B15" s="18">
+      <c r="B16" s="18">
         <v>530.5</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="D16" s="94" t="s">
+        <v>430</v>
+      </c>
+      <c r="E16" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F16" s="96">
+        <v>790.4</v>
+      </c>
+      <c r="G16" s="96">
+        <v>775.3</v>
+      </c>
+      <c r="J16" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>325</v>
       </c>
-      <c r="B16" s="18">
+      <c r="B17" s="18">
         <v>465.4</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="16" t="s">
+      <c r="D17" s="94" t="s">
+        <v>431</v>
+      </c>
+      <c r="E17" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F17" s="96">
+        <v>697</v>
+      </c>
+      <c r="G17" s="96">
+        <v>695.1</v>
+      </c>
+      <c r="J17" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="16" t="s">
         <v>339</v>
       </c>
-      <c r="B17" s="18">
+      <c r="B18" s="18">
         <v>424.3</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="16" t="s">
+      <c r="D18" s="94" t="s">
+        <v>432</v>
+      </c>
+      <c r="E18" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F18" s="96">
+        <v>714.4</v>
+      </c>
+      <c r="G18" s="96">
+        <v>696.3</v>
+      </c>
+      <c r="J18" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="16" t="s">
         <v>340</v>
       </c>
-      <c r="B18" s="18">
+      <c r="B19" s="18">
         <v>397.3</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="16" t="s">
+      <c r="D19" s="94" t="s">
+        <v>433</v>
+      </c>
+      <c r="E19" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F19" s="96">
+        <v>636.9</v>
+      </c>
+      <c r="G19" s="96">
+        <v>614.79999999999995</v>
+      </c>
+      <c r="J19" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="16" t="s">
         <v>341</v>
       </c>
-      <c r="B19" s="18">
+      <c r="B20" s="18">
         <v>441.3</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="16" t="s">
+      <c r="D20" s="94" t="s">
+        <v>434</v>
+      </c>
+      <c r="E20" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F20" s="96">
+        <v>990.1</v>
+      </c>
+      <c r="G20" s="96">
+        <v>850</v>
+      </c>
+      <c r="J20" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="16" t="s">
         <v>342</v>
       </c>
-      <c r="B20" s="18">
+      <c r="B21" s="18">
         <v>444.1</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="16" t="s">
+      <c r="D21" s="94" t="s">
+        <v>435</v>
+      </c>
+      <c r="E21" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F21" s="96">
+        <v>840.1</v>
+      </c>
+      <c r="G21" s="96">
+        <v>721.8</v>
+      </c>
+      <c r="J21" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B22" s="18">
         <v>428.8</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="17" t="s">
+      <c r="D22" s="94" t="s">
+        <v>436</v>
+      </c>
+      <c r="E22" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F22" s="96">
+        <v>737</v>
+      </c>
+      <c r="G22" s="96">
+        <v>645.20000000000005</v>
+      </c>
+      <c r="J22" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="17" t="s">
         <v>344</v>
       </c>
-      <c r="B22" s="20">
+      <c r="B23" s="20">
         <v>393</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="D23" s="94" t="s">
+        <v>437</v>
+      </c>
+      <c r="E23" s="95" t="s">
+        <v>403</v>
+      </c>
+      <c r="F23" s="96">
+        <v>545.79999999999995</v>
+      </c>
+      <c r="G23" s="96">
+        <v>545.79999999999995</v>
+      </c>
+      <c r="J23" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>331</v>
       </c>
-      <c r="B23" s="18">
+      <c r="B24" s="18">
         <v>461.1</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="D24" s="97" t="s">
+        <v>438</v>
+      </c>
+      <c r="E24" s="98" t="s">
+        <v>408</v>
+      </c>
+      <c r="F24" s="99">
+        <v>885.6</v>
+      </c>
+      <c r="G24" s="99">
+        <v>761.5</v>
+      </c>
+      <c r="J24" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>332</v>
       </c>
-      <c r="B24" s="18">
+      <c r="B25" s="18">
         <v>351.8</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="D25" s="97" t="s">
+        <v>439</v>
+      </c>
+      <c r="E25" s="98" t="s">
+        <v>408</v>
+      </c>
+      <c r="F25" s="99">
+        <v>741.4</v>
+      </c>
+      <c r="G25" s="99">
+        <v>664.4</v>
+      </c>
+      <c r="J25" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>333</v>
       </c>
-      <c r="B25" s="18">
+      <c r="B26" s="18">
         <v>332.8</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="D26" s="97" t="s">
+        <v>440</v>
+      </c>
+      <c r="E26" s="98" t="s">
+        <v>408</v>
+      </c>
+      <c r="F26" s="99">
+        <v>642.70000000000005</v>
+      </c>
+      <c r="G26" s="99">
+        <v>603.5</v>
+      </c>
+      <c r="J26" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>334</v>
       </c>
-      <c r="B26" s="18">
+      <c r="B27" s="18">
         <v>306.60000000000002</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="D27" s="97" t="s">
+        <v>441</v>
+      </c>
+      <c r="E27" s="98" t="s">
+        <v>408</v>
+      </c>
+      <c r="F27" s="99">
+        <v>598.1</v>
+      </c>
+      <c r="G27" s="99">
+        <v>541.1</v>
+      </c>
+      <c r="J27" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>335</v>
       </c>
-      <c r="B27" s="18">
+      <c r="B28" s="18">
         <v>411.3</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+      <c r="D28" s="97" t="s">
+        <v>442</v>
+      </c>
+      <c r="E28" s="98" t="s">
+        <v>408</v>
+      </c>
+      <c r="F28" s="99">
+        <v>1223.2</v>
+      </c>
+      <c r="G28" s="99">
+        <v>1164.4000000000001</v>
+      </c>
+      <c r="J28" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>336</v>
       </c>
-      <c r="B28" s="18">
+      <c r="B29" s="18">
         <v>345.5</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+      <c r="D29" s="97" t="s">
+        <v>443</v>
+      </c>
+      <c r="E29" s="98" t="s">
+        <v>408</v>
+      </c>
+      <c r="F29" s="99">
+        <v>1083.0999999999999</v>
+      </c>
+      <c r="G29" s="99">
+        <v>1041.2</v>
+      </c>
+      <c r="J29" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
         <v>337</v>
       </c>
-      <c r="B29" s="18">
+      <c r="B30" s="18">
         <v>298.3</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+      <c r="D30" s="97" t="s">
+        <v>444</v>
+      </c>
+      <c r="E30" s="98" t="s">
+        <v>408</v>
+      </c>
+      <c r="F30" s="99">
+        <v>1083.0999999999999</v>
+      </c>
+      <c r="G30" s="99">
+        <v>1041.2</v>
+      </c>
+      <c r="J30" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
         <v>338</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B31" s="15">
         <v>294.5</v>
+      </c>
+      <c r="D31" s="97" t="s">
+        <v>445</v>
+      </c>
+      <c r="E31" s="98" t="s">
+        <v>408</v>
+      </c>
+      <c r="F31" s="99">
+        <v>1081.0999999999999</v>
+      </c>
+      <c r="G31" s="99">
+        <v>1001.2</v>
+      </c>
+      <c r="J31" t="s">
+        <v>489</v>
       </c>
     </row>
   </sheetData>

</xml_diff>